<commit_message>
Build הגדרות (Settings) sheet with 9 named-range tables
Populates the Settings sheet as the single source of truth for all
dropdowns: Environments, Prints, Product Lines, Products, Fabric Types,
Statuses, Yes/No, Sizes, and SKU mapping. All tables are styled with
dark headers, alternating row colors, RTL direction, and registered
as Named Ranges for cross-sheet reference.

https://claude.ai/code/session_01UnayhTNE4ZcMSuocT9bjvX
</commit_message>
<xml_diff>
--- a/ametrine_inventory.xlsx
+++ b/ametrine_inventory.xlsx
@@ -16,7 +16,17 @@
     <sheet name="הגדרות" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="מלאי רצוי" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="סביבות">'הגדרות'!$A$2:$A$7</definedName>
+    <definedName name="הדפסים">'הגדרות'!$A$11:$D$25</definedName>
+    <definedName name="קווי_מוצר">'הגדרות'!$A$29:$A$36</definedName>
+    <definedName name="מוצרים">'הגדרות'!$A$40:$C$63</definedName>
+    <definedName name="סוגי_בד">'הגדרות'!$A$67:$A$78</definedName>
+    <definedName name="סטטוסים">'הגדרות'!$A$82:$A$85</definedName>
+    <definedName name="כן_לא">'הגדרות'!$A$89:$A$90</definedName>
+    <definedName name="מידות">'הגדרות'!$A$94:$A$100</definedName>
+    <definedName name="מקטים">'הגדרות'!$A$104:$D$123</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -24,7 +34,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +42,39 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+        <bgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +82,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B0B0B0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B0B0B0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B0B0B0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B0B0B0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -498,9 +554,1038 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>סביבה</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>מדברי</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>מיוער</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>שלג</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ימי</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>מבולדר/שטח בנוי</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>אחר</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>הדפס</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>סביבה ראשית</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>סביבה משנית</t>
+        </is>
+      </c>
+      <c r="D10" s="1" t="inlineStr">
+        <is>
+          <t>תמונה</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Desert</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>מדברי</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Desert-Green</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>מדברי</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n"/>
+      <c r="D12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Desert Coyote</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>מדברי</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Sand</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>מדברי</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n"/>
+      <c r="D14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Ever-Green</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>מיוער</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Forest Green</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>מיוער</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Kestrel</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>מיוער</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Woodland</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>מיוער</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n"/>
+      <c r="D18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Woodland Brown</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>מיוער</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Urban Green</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>מיוער</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>מבולדר/שטח בנוי</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Snirt Snow</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>שלג</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Fresh Snow</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>שלג</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Marine</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>ימי</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>מבולדר/שטח בנוי</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Boulder</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>מבולדר/שטח בנוי</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
+        <is>
+          <t>קו מוצר</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Hide Site</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Platform Hide Site</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Uniform</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Blankets</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Platform On-The-Move</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>קו מוצר</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
+          <t>שם מוצר</t>
+        </is>
+      </c>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>גרסאות זמינות</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Hobey Elite</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Gal Suit</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Sniper Assault</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>SWAT 3-Part Suit</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>May Suit</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>May Long Shirt</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Arctic Suit</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Poncho SRV</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Poncho Inbar</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Poncho Inbar 3D</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Poncho Sahar</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>OverGarment</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Poncho Sahar 3D</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Hide Site</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Hide Site Standard</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Hide Site</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>HS Floor</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Hide Site</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Window Kit</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Platform Hide Site</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Platform HS (including parts)</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Uniform</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Shirt</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Uniform</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Pants</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Blankets</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Survival Blanket</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Blankets</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>יריעת החשכה</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Urban</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Loki</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>Platform On-The-Move</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>GMV</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Platform On-The-Move</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>רשת הצללה</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>Accessories</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr">
+        <is>
+          <t>סוג בד</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Sahar</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Inbar</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>SRV</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Gabardine</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Meron</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Arber</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>IRR</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Polar</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Nylon</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Mesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr">
+        <is>
+          <t>סטטוס</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>במלאי</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>מושאל</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>בחדר תצוגה</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>בתיק הדגמה</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="inlineStr">
+        <is>
+          <t>ערך</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>כן</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>לא</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="inlineStr">
+        <is>
+          <t>מידה</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>XXL</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>One Size</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="inlineStr">
+        <is>
+          <t>מוצר</t>
+        </is>
+      </c>
+      <c r="B103" s="1" t="inlineStr">
+        <is>
+          <t>סוג בד</t>
+        </is>
+      </c>
+      <c r="C103" s="1" t="inlineStr">
+        <is>
+          <t>גרסה</t>
+        </is>
+      </c>
+      <c r="D103" s="1" t="inlineStr">
+        <is>
+          <t>מק"ט</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr"/>
+      <c r="B104" s="2" t="inlineStr"/>
+      <c r="C104" s="2" t="inlineStr"/>
+      <c r="D104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr"/>
+      <c r="B105" s="3" t="inlineStr"/>
+      <c r="C105" s="3" t="inlineStr"/>
+      <c r="D105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr"/>
+      <c r="B106" s="2" t="inlineStr"/>
+      <c r="C106" s="2" t="inlineStr"/>
+      <c r="D106" s="2" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr"/>
+      <c r="B107" s="3" t="inlineStr"/>
+      <c r="C107" s="3" t="inlineStr"/>
+      <c r="D107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr"/>
+      <c r="B108" s="2" t="inlineStr"/>
+      <c r="C108" s="2" t="inlineStr"/>
+      <c r="D108" s="2" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr"/>
+      <c r="B109" s="3" t="inlineStr"/>
+      <c r="C109" s="3" t="inlineStr"/>
+      <c r="D109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr"/>
+      <c r="B110" s="2" t="inlineStr"/>
+      <c r="C110" s="2" t="inlineStr"/>
+      <c r="D110" s="2" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr"/>
+      <c r="B111" s="3" t="inlineStr"/>
+      <c r="C111" s="3" t="inlineStr"/>
+      <c r="D111" s="3" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr"/>
+      <c r="B112" s="2" t="inlineStr"/>
+      <c r="C112" s="2" t="inlineStr"/>
+      <c r="D112" s="2" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr"/>
+      <c r="B113" s="3" t="inlineStr"/>
+      <c r="C113" s="3" t="inlineStr"/>
+      <c r="D113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr"/>
+      <c r="B114" s="2" t="inlineStr"/>
+      <c r="C114" s="2" t="inlineStr"/>
+      <c r="D114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr"/>
+      <c r="B115" s="3" t="inlineStr"/>
+      <c r="C115" s="3" t="inlineStr"/>
+      <c r="D115" s="3" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr"/>
+      <c r="B116" s="2" t="inlineStr"/>
+      <c r="C116" s="2" t="inlineStr"/>
+      <c r="D116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr"/>
+      <c r="B117" s="3" t="inlineStr"/>
+      <c r="C117" s="3" t="inlineStr"/>
+      <c r="D117" s="3" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr"/>
+      <c r="B118" s="2" t="inlineStr"/>
+      <c r="C118" s="2" t="inlineStr"/>
+      <c r="D118" s="2" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr"/>
+      <c r="B119" s="3" t="inlineStr"/>
+      <c r="C119" s="3" t="inlineStr"/>
+      <c r="D119" s="3" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr"/>
+      <c r="B120" s="2" t="inlineStr"/>
+      <c r="C120" s="2" t="inlineStr"/>
+      <c r="D120" s="2" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr"/>
+      <c r="B121" s="3" t="inlineStr"/>
+      <c r="C121" s="3" t="inlineStr"/>
+      <c r="D121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr"/>
+      <c r="B122" s="2" t="inlineStr"/>
+      <c r="C122" s="2" t="inlineStr"/>
+      <c r="D122" s="2" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr"/>
+      <c r="B123" s="3" t="inlineStr"/>
+      <c r="C123" s="3" t="inlineStr"/>
+      <c r="D123" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Build השאלות (Loans) sheet with filtered view of loaned items
- Filter area (rows 1-2): dropdown filters for country, loaned-to,
  company contact, and overdue status (Yes/No)
- Display table (rows 4-104): auto-pulls all inventory rows where
  status=מושאל using SMALL/IF array formulas with INDEX lookups
- Hidden helper column K computes nth matching row index with all
  filter conditions applied
- Overdue detection: shows "באיחור!" with red bold font when
  expected return < TODAY()
- Conditional formatting: red highlight on entire row for overdue items
- RTL, dark headers, alternating rows, frozen header, 100 display rows

https://claude.ai/code/session_01UnayhTNE4ZcMSuocT9bjvX
</commit_message>
<xml_diff>
--- a/ametrine_inventory.xlsx
+++ b/ametrine_inventory.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -129,16 +129,39 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFFF00"/>
           <bgColor rgb="00FFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+          <bgColor rgb="00FFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -23214,9 +23237,4723 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
+    <col hidden="1" width="10" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>מדינה</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>מושאל ל</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>אחראי מהחברה</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>באיחור</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="n"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>מזהה ייחודי</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>שם מוצר</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>גרסה</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>מושאל ל</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>מדינה</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>אחראי מהחברה</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>תאריך השאלה</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>החזרה משוערת</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>באיחור</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>הערות</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>row_ref</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <f>IF($K5="","",INDEX(מלאי!$D$2:$D$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="B5" s="2">
+        <f>IF($K5="","",INDEX(מלאי!$B$2:$B$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="C5" s="2">
+        <f>IF($K5="","",INDEX(מלאי!$C$2:$C$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="D5" s="2">
+        <f>IF($K5="","",INDEX(מלאי!$Y$2:$Y$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="E5" s="2">
+        <f>IF($K5="","",INDEX(מלאי!$Z$2:$Z$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="F5" s="2">
+        <f>IF($K5="","",INDEX(מלאי!$AA$2:$AA$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="G5" s="3">
+        <f>IF($K5="","",INDEX(מלאי!$F$2:$F$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="H5" s="3">
+        <f>IF($K5="","",INDEX(מלאי!$AB$2:$AB$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="I5" s="2">
+        <f>IF($K5="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K5)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K5)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J5" s="2">
+        <f>IF($K5="","",INDEX(מלאי!$AC$2:$AC$500,$K5))</f>
+        <v/>
+      </c>
+      <c r="K5" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),1),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4">
+        <f>IF($K6="","",INDEX(מלאי!$D$2:$D$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="B6" s="4">
+        <f>IF($K6="","",INDEX(מלאי!$B$2:$B$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
+        <f>IF($K6="","",INDEX(מלאי!$C$2:$C$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>IF($K6="","",INDEX(מלאי!$Y$2:$Y$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>IF($K6="","",INDEX(מלאי!$Z$2:$Z$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>IF($K6="","",INDEX(מלאי!$AA$2:$AA$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>IF($K6="","",INDEX(מלאי!$F$2:$F$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>IF($K6="","",INDEX(מלאי!$AB$2:$AB$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="I6" s="4">
+        <f>IF($K6="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K6)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K6)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J6" s="4">
+        <f>IF($K6="","",INDEX(מלאי!$AC$2:$AC$500,$K6))</f>
+        <v/>
+      </c>
+      <c r="K6" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),2),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <f>IF($K7="","",INDEX(מלאי!$D$2:$D$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="B7" s="2">
+        <f>IF($K7="","",INDEX(מלאי!$B$2:$B$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="C7" s="2">
+        <f>IF($K7="","",INDEX(מלאי!$C$2:$C$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="D7" s="2">
+        <f>IF($K7="","",INDEX(מלאי!$Y$2:$Y$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="E7" s="2">
+        <f>IF($K7="","",INDEX(מלאי!$Z$2:$Z$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="F7" s="2">
+        <f>IF($K7="","",INDEX(מלאי!$AA$2:$AA$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="G7" s="3">
+        <f>IF($K7="","",INDEX(מלאי!$F$2:$F$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="H7" s="3">
+        <f>IF($K7="","",INDEX(מלאי!$AB$2:$AB$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="I7" s="2">
+        <f>IF($K7="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K7)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K7)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J7" s="2">
+        <f>IF($K7="","",INDEX(מלאי!$AC$2:$AC$500,$K7))</f>
+        <v/>
+      </c>
+      <c r="K7" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),3),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4">
+        <f>IF($K8="","",INDEX(מלאי!$D$2:$D$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="B8" s="4">
+        <f>IF($K8="","",INDEX(מלאי!$B$2:$B$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
+        <f>IF($K8="","",INDEX(מלאי!$C$2:$C$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>IF($K8="","",INDEX(מלאי!$Y$2:$Y$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>IF($K8="","",INDEX(מלאי!$Z$2:$Z$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>IF($K8="","",INDEX(מלאי!$AA$2:$AA$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>IF($K8="","",INDEX(מלאי!$F$2:$F$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>IF($K8="","",INDEX(מלאי!$AB$2:$AB$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>IF($K8="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K8)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K8)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J8" s="4">
+        <f>IF($K8="","",INDEX(מלאי!$AC$2:$AC$500,$K8))</f>
+        <v/>
+      </c>
+      <c r="K8" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),4),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <f>IF($K9="","",INDEX(מלאי!$D$2:$D$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="B9" s="2">
+        <f>IF($K9="","",INDEX(מלאי!$B$2:$B$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="C9" s="2">
+        <f>IF($K9="","",INDEX(מלאי!$C$2:$C$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="D9" s="2">
+        <f>IF($K9="","",INDEX(מלאי!$Y$2:$Y$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="E9" s="2">
+        <f>IF($K9="","",INDEX(מלאי!$Z$2:$Z$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="F9" s="2">
+        <f>IF($K9="","",INDEX(מלאי!$AA$2:$AA$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="G9" s="3">
+        <f>IF($K9="","",INDEX(מלאי!$F$2:$F$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="H9" s="3">
+        <f>IF($K9="","",INDEX(מלאי!$AB$2:$AB$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="I9" s="2">
+        <f>IF($K9="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K9)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K9)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J9" s="2">
+        <f>IF($K9="","",INDEX(מלאי!$AC$2:$AC$500,$K9))</f>
+        <v/>
+      </c>
+      <c r="K9" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),5),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4">
+        <f>IF($K10="","",INDEX(מלאי!$D$2:$D$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="B10" s="4">
+        <f>IF($K10="","",INDEX(מלאי!$B$2:$B$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="C10" s="4">
+        <f>IF($K10="","",INDEX(מלאי!$C$2:$C$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
+        <f>IF($K10="","",INDEX(מלאי!$Y$2:$Y$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>IF($K10="","",INDEX(מלאי!$Z$2:$Z$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>IF($K10="","",INDEX(מלאי!$AA$2:$AA$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>IF($K10="","",INDEX(מלאי!$F$2:$F$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>IF($K10="","",INDEX(מלאי!$AB$2:$AB$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="I10" s="4">
+        <f>IF($K10="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K10)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K10)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J10" s="4">
+        <f>IF($K10="","",INDEX(מלאי!$AC$2:$AC$500,$K10))</f>
+        <v/>
+      </c>
+      <c r="K10" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),6),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <f>IF($K11="","",INDEX(מלאי!$D$2:$D$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="B11" s="2">
+        <f>IF($K11="","",INDEX(מלאי!$B$2:$B$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="C11" s="2">
+        <f>IF($K11="","",INDEX(מלאי!$C$2:$C$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="D11" s="2">
+        <f>IF($K11="","",INDEX(מלאי!$Y$2:$Y$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="E11" s="2">
+        <f>IF($K11="","",INDEX(מלאי!$Z$2:$Z$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="F11" s="2">
+        <f>IF($K11="","",INDEX(מלאי!$AA$2:$AA$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="G11" s="3">
+        <f>IF($K11="","",INDEX(מלאי!$F$2:$F$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="H11" s="3">
+        <f>IF($K11="","",INDEX(מלאי!$AB$2:$AB$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="I11" s="2">
+        <f>IF($K11="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K11)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K11)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J11" s="2">
+        <f>IF($K11="","",INDEX(מלאי!$AC$2:$AC$500,$K11))</f>
+        <v/>
+      </c>
+      <c r="K11" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),7),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4">
+        <f>IF($K12="","",INDEX(מלאי!$D$2:$D$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="B12" s="4">
+        <f>IF($K12="","",INDEX(מלאי!$B$2:$B$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="C12" s="4">
+        <f>IF($K12="","",INDEX(מלאי!$C$2:$C$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
+        <f>IF($K12="","",INDEX(מלאי!$Y$2:$Y$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="E12" s="4">
+        <f>IF($K12="","",INDEX(מלאי!$Z$2:$Z$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="F12" s="4">
+        <f>IF($K12="","",INDEX(מלאי!$AA$2:$AA$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>IF($K12="","",INDEX(מלאי!$F$2:$F$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="H12" s="5">
+        <f>IF($K12="","",INDEX(מלאי!$AB$2:$AB$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="I12" s="4">
+        <f>IF($K12="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K12)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K12)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J12" s="4">
+        <f>IF($K12="","",INDEX(מלאי!$AC$2:$AC$500,$K12))</f>
+        <v/>
+      </c>
+      <c r="K12" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),8),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
+        <f>IF($K13="","",INDEX(מלאי!$D$2:$D$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="B13" s="2">
+        <f>IF($K13="","",INDEX(מלאי!$B$2:$B$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="C13" s="2">
+        <f>IF($K13="","",INDEX(מלאי!$C$2:$C$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="D13" s="2">
+        <f>IF($K13="","",INDEX(מלאי!$Y$2:$Y$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="E13" s="2">
+        <f>IF($K13="","",INDEX(מלאי!$Z$2:$Z$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="F13" s="2">
+        <f>IF($K13="","",INDEX(מלאי!$AA$2:$AA$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="G13" s="3">
+        <f>IF($K13="","",INDEX(מלאי!$F$2:$F$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="H13" s="3">
+        <f>IF($K13="","",INDEX(מלאי!$AB$2:$AB$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="I13" s="2">
+        <f>IF($K13="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K13)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K13)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J13" s="2">
+        <f>IF($K13="","",INDEX(מלאי!$AC$2:$AC$500,$K13))</f>
+        <v/>
+      </c>
+      <c r="K13" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),9),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4">
+        <f>IF($K14="","",INDEX(מלאי!$D$2:$D$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="B14" s="4">
+        <f>IF($K14="","",INDEX(מלאי!$B$2:$B$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="C14" s="4">
+        <f>IF($K14="","",INDEX(מלאי!$C$2:$C$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="D14" s="4">
+        <f>IF($K14="","",INDEX(מלאי!$Y$2:$Y$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="E14" s="4">
+        <f>IF($K14="","",INDEX(מלאי!$Z$2:$Z$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="F14" s="4">
+        <f>IF($K14="","",INDEX(מלאי!$AA$2:$AA$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="G14" s="5">
+        <f>IF($K14="","",INDEX(מלאי!$F$2:$F$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="H14" s="5">
+        <f>IF($K14="","",INDEX(מלאי!$AB$2:$AB$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="I14" s="4">
+        <f>IF($K14="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K14)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K14)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J14" s="4">
+        <f>IF($K14="","",INDEX(מלאי!$AC$2:$AC$500,$K14))</f>
+        <v/>
+      </c>
+      <c r="K14" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),10),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <f>IF($K15="","",INDEX(מלאי!$D$2:$D$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="B15" s="2">
+        <f>IF($K15="","",INDEX(מלאי!$B$2:$B$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="C15" s="2">
+        <f>IF($K15="","",INDEX(מלאי!$C$2:$C$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="D15" s="2">
+        <f>IF($K15="","",INDEX(מלאי!$Y$2:$Y$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="E15" s="2">
+        <f>IF($K15="","",INDEX(מלאי!$Z$2:$Z$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="F15" s="2">
+        <f>IF($K15="","",INDEX(מלאי!$AA$2:$AA$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="G15" s="3">
+        <f>IF($K15="","",INDEX(מלאי!$F$2:$F$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="H15" s="3">
+        <f>IF($K15="","",INDEX(מלאי!$AB$2:$AB$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="I15" s="2">
+        <f>IF($K15="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K15)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K15)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J15" s="2">
+        <f>IF($K15="","",INDEX(מלאי!$AC$2:$AC$500,$K15))</f>
+        <v/>
+      </c>
+      <c r="K15" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),11),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4">
+        <f>IF($K16="","",INDEX(מלאי!$D$2:$D$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="B16" s="4">
+        <f>IF($K16="","",INDEX(מלאי!$B$2:$B$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="C16" s="4">
+        <f>IF($K16="","",INDEX(מלאי!$C$2:$C$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="D16" s="4">
+        <f>IF($K16="","",INDEX(מלאי!$Y$2:$Y$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="E16" s="4">
+        <f>IF($K16="","",INDEX(מלאי!$Z$2:$Z$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="F16" s="4">
+        <f>IF($K16="","",INDEX(מלאי!$AA$2:$AA$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="G16" s="5">
+        <f>IF($K16="","",INDEX(מלאי!$F$2:$F$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="H16" s="5">
+        <f>IF($K16="","",INDEX(מלאי!$AB$2:$AB$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="I16" s="4">
+        <f>IF($K16="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K16)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K16)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J16" s="4">
+        <f>IF($K16="","",INDEX(מלאי!$AC$2:$AC$500,$K16))</f>
+        <v/>
+      </c>
+      <c r="K16" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
+        <f>IF($K17="","",INDEX(מלאי!$D$2:$D$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="B17" s="2">
+        <f>IF($K17="","",INDEX(מלאי!$B$2:$B$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="C17" s="2">
+        <f>IF($K17="","",INDEX(מלאי!$C$2:$C$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="D17" s="2">
+        <f>IF($K17="","",INDEX(מלאי!$Y$2:$Y$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="E17" s="2">
+        <f>IF($K17="","",INDEX(מלאי!$Z$2:$Z$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="F17" s="2">
+        <f>IF($K17="","",INDEX(מלאי!$AA$2:$AA$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="G17" s="3">
+        <f>IF($K17="","",INDEX(מלאי!$F$2:$F$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="H17" s="3">
+        <f>IF($K17="","",INDEX(מלאי!$AB$2:$AB$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="I17" s="2">
+        <f>IF($K17="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K17)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K17)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J17" s="2">
+        <f>IF($K17="","",INDEX(מלאי!$AC$2:$AC$500,$K17))</f>
+        <v/>
+      </c>
+      <c r="K17" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4">
+        <f>IF($K18="","",INDEX(מלאי!$D$2:$D$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="B18" s="4">
+        <f>IF($K18="","",INDEX(מלאי!$B$2:$B$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="C18" s="4">
+        <f>IF($K18="","",INDEX(מלאי!$C$2:$C$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="D18" s="4">
+        <f>IF($K18="","",INDEX(מלאי!$Y$2:$Y$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="E18" s="4">
+        <f>IF($K18="","",INDEX(מלאי!$Z$2:$Z$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="F18" s="4">
+        <f>IF($K18="","",INDEX(מלאי!$AA$2:$AA$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="G18" s="5">
+        <f>IF($K18="","",INDEX(מלאי!$F$2:$F$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="H18" s="5">
+        <f>IF($K18="","",INDEX(מלאי!$AB$2:$AB$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="I18" s="4">
+        <f>IF($K18="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K18)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K18)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J18" s="4">
+        <f>IF($K18="","",INDEX(מלאי!$AC$2:$AC$500,$K18))</f>
+        <v/>
+      </c>
+      <c r="K18" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2">
+        <f>IF($K19="","",INDEX(מלאי!$D$2:$D$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="B19" s="2">
+        <f>IF($K19="","",INDEX(מלאי!$B$2:$B$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="C19" s="2">
+        <f>IF($K19="","",INDEX(מלאי!$C$2:$C$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="D19" s="2">
+        <f>IF($K19="","",INDEX(מלאי!$Y$2:$Y$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="E19" s="2">
+        <f>IF($K19="","",INDEX(מלאי!$Z$2:$Z$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="F19" s="2">
+        <f>IF($K19="","",INDEX(מלאי!$AA$2:$AA$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="G19" s="3">
+        <f>IF($K19="","",INDEX(מלאי!$F$2:$F$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="H19" s="3">
+        <f>IF($K19="","",INDEX(מלאי!$AB$2:$AB$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="I19" s="2">
+        <f>IF($K19="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K19)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K19)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J19" s="2">
+        <f>IF($K19="","",INDEX(מלאי!$AC$2:$AC$500,$K19))</f>
+        <v/>
+      </c>
+      <c r="K19" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4">
+        <f>IF($K20="","",INDEX(מלאי!$D$2:$D$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="B20" s="4">
+        <f>IF($K20="","",INDEX(מלאי!$B$2:$B$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="C20" s="4">
+        <f>IF($K20="","",INDEX(מלאי!$C$2:$C$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="D20" s="4">
+        <f>IF($K20="","",INDEX(מלאי!$Y$2:$Y$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="E20" s="4">
+        <f>IF($K20="","",INDEX(מלאי!$Z$2:$Z$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="F20" s="4">
+        <f>IF($K20="","",INDEX(מלאי!$AA$2:$AA$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="G20" s="5">
+        <f>IF($K20="","",INDEX(מלאי!$F$2:$F$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="H20" s="5">
+        <f>IF($K20="","",INDEX(מלאי!$AB$2:$AB$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="I20" s="4">
+        <f>IF($K20="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K20)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K20)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J20" s="4">
+        <f>IF($K20="","",INDEX(מלאי!$AC$2:$AC$500,$K20))</f>
+        <v/>
+      </c>
+      <c r="K20" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2">
+        <f>IF($K21="","",INDEX(מלאי!$D$2:$D$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="B21" s="2">
+        <f>IF($K21="","",INDEX(מלאי!$B$2:$B$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="C21" s="2">
+        <f>IF($K21="","",INDEX(מלאי!$C$2:$C$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="D21" s="2">
+        <f>IF($K21="","",INDEX(מלאי!$Y$2:$Y$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="E21" s="2">
+        <f>IF($K21="","",INDEX(מלאי!$Z$2:$Z$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="F21" s="2">
+        <f>IF($K21="","",INDEX(מלאי!$AA$2:$AA$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="G21" s="3">
+        <f>IF($K21="","",INDEX(מלאי!$F$2:$F$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="H21" s="3">
+        <f>IF($K21="","",INDEX(מלאי!$AB$2:$AB$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="I21" s="2">
+        <f>IF($K21="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K21)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K21)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J21" s="2">
+        <f>IF($K21="","",INDEX(מלאי!$AC$2:$AC$500,$K21))</f>
+        <v/>
+      </c>
+      <c r="K21" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4">
+        <f>IF($K22="","",INDEX(מלאי!$D$2:$D$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="B22" s="4">
+        <f>IF($K22="","",INDEX(מלאי!$B$2:$B$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="C22" s="4">
+        <f>IF($K22="","",INDEX(מלאי!$C$2:$C$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="D22" s="4">
+        <f>IF($K22="","",INDEX(מלאי!$Y$2:$Y$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="E22" s="4">
+        <f>IF($K22="","",INDEX(מלאי!$Z$2:$Z$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="F22" s="4">
+        <f>IF($K22="","",INDEX(מלאי!$AA$2:$AA$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="G22" s="5">
+        <f>IF($K22="","",INDEX(מלאי!$F$2:$F$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="H22" s="5">
+        <f>IF($K22="","",INDEX(מלאי!$AB$2:$AB$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="I22" s="4">
+        <f>IF($K22="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K22)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K22)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J22" s="4">
+        <f>IF($K22="","",INDEX(מלאי!$AC$2:$AC$500,$K22))</f>
+        <v/>
+      </c>
+      <c r="K22" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2">
+        <f>IF($K23="","",INDEX(מלאי!$D$2:$D$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="B23" s="2">
+        <f>IF($K23="","",INDEX(מלאי!$B$2:$B$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="C23" s="2">
+        <f>IF($K23="","",INDEX(מלאי!$C$2:$C$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="D23" s="2">
+        <f>IF($K23="","",INDEX(מלאי!$Y$2:$Y$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="E23" s="2">
+        <f>IF($K23="","",INDEX(מלאי!$Z$2:$Z$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="F23" s="2">
+        <f>IF($K23="","",INDEX(מלאי!$AA$2:$AA$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="G23" s="3">
+        <f>IF($K23="","",INDEX(מלאי!$F$2:$F$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="H23" s="3">
+        <f>IF($K23="","",INDEX(מלאי!$AB$2:$AB$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="I23" s="2">
+        <f>IF($K23="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K23)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K23)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J23" s="2">
+        <f>IF($K23="","",INDEX(מלאי!$AC$2:$AC$500,$K23))</f>
+        <v/>
+      </c>
+      <c r="K23" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4">
+        <f>IF($K24="","",INDEX(מלאי!$D$2:$D$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="B24" s="4">
+        <f>IF($K24="","",INDEX(מלאי!$B$2:$B$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="C24" s="4">
+        <f>IF($K24="","",INDEX(מלאי!$C$2:$C$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="D24" s="4">
+        <f>IF($K24="","",INDEX(מלאי!$Y$2:$Y$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="E24" s="4">
+        <f>IF($K24="","",INDEX(מלאי!$Z$2:$Z$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="F24" s="4">
+        <f>IF($K24="","",INDEX(מלאי!$AA$2:$AA$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="G24" s="5">
+        <f>IF($K24="","",INDEX(מלאי!$F$2:$F$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="H24" s="5">
+        <f>IF($K24="","",INDEX(מלאי!$AB$2:$AB$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="I24" s="4">
+        <f>IF($K24="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K24)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K24)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J24" s="4">
+        <f>IF($K24="","",INDEX(מלאי!$AC$2:$AC$500,$K24))</f>
+        <v/>
+      </c>
+      <c r="K24" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
+        <f>IF($K25="","",INDEX(מלאי!$D$2:$D$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="B25" s="2">
+        <f>IF($K25="","",INDEX(מלאי!$B$2:$B$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="C25" s="2">
+        <f>IF($K25="","",INDEX(מלאי!$C$2:$C$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="D25" s="2">
+        <f>IF($K25="","",INDEX(מלאי!$Y$2:$Y$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="E25" s="2">
+        <f>IF($K25="","",INDEX(מלאי!$Z$2:$Z$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="F25" s="2">
+        <f>IF($K25="","",INDEX(מלאי!$AA$2:$AA$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="G25" s="3">
+        <f>IF($K25="","",INDEX(מלאי!$F$2:$F$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="H25" s="3">
+        <f>IF($K25="","",INDEX(מלאי!$AB$2:$AB$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="I25" s="2">
+        <f>IF($K25="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K25)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K25)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J25" s="2">
+        <f>IF($K25="","",INDEX(מלאי!$AC$2:$AC$500,$K25))</f>
+        <v/>
+      </c>
+      <c r="K25" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4">
+        <f>IF($K26="","",INDEX(מלאי!$D$2:$D$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="B26" s="4">
+        <f>IF($K26="","",INDEX(מלאי!$B$2:$B$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="C26" s="4">
+        <f>IF($K26="","",INDEX(מלאי!$C$2:$C$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="D26" s="4">
+        <f>IF($K26="","",INDEX(מלאי!$Y$2:$Y$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="E26" s="4">
+        <f>IF($K26="","",INDEX(מלאי!$Z$2:$Z$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="F26" s="4">
+        <f>IF($K26="","",INDEX(מלאי!$AA$2:$AA$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="G26" s="5">
+        <f>IF($K26="","",INDEX(מלאי!$F$2:$F$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="H26" s="5">
+        <f>IF($K26="","",INDEX(מלאי!$AB$2:$AB$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="I26" s="4">
+        <f>IF($K26="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K26)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K26)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J26" s="4">
+        <f>IF($K26="","",INDEX(מלאי!$AC$2:$AC$500,$K26))</f>
+        <v/>
+      </c>
+      <c r="K26" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2">
+        <f>IF($K27="","",INDEX(מלאי!$D$2:$D$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="B27" s="2">
+        <f>IF($K27="","",INDEX(מלאי!$B$2:$B$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="C27" s="2">
+        <f>IF($K27="","",INDEX(מלאי!$C$2:$C$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="D27" s="2">
+        <f>IF($K27="","",INDEX(מלאי!$Y$2:$Y$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="E27" s="2">
+        <f>IF($K27="","",INDEX(מלאי!$Z$2:$Z$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="F27" s="2">
+        <f>IF($K27="","",INDEX(מלאי!$AA$2:$AA$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="G27" s="3">
+        <f>IF($K27="","",INDEX(מלאי!$F$2:$F$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="H27" s="3">
+        <f>IF($K27="","",INDEX(מלאי!$AB$2:$AB$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="I27" s="2">
+        <f>IF($K27="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K27)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K27)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J27" s="2">
+        <f>IF($K27="","",INDEX(מלאי!$AC$2:$AC$500,$K27))</f>
+        <v/>
+      </c>
+      <c r="K27" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4">
+        <f>IF($K28="","",INDEX(מלאי!$D$2:$D$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="B28" s="4">
+        <f>IF($K28="","",INDEX(מלאי!$B$2:$B$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="C28" s="4">
+        <f>IF($K28="","",INDEX(מלאי!$C$2:$C$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="D28" s="4">
+        <f>IF($K28="","",INDEX(מלאי!$Y$2:$Y$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="E28" s="4">
+        <f>IF($K28="","",INDEX(מלאי!$Z$2:$Z$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="F28" s="4">
+        <f>IF($K28="","",INDEX(מלאי!$AA$2:$AA$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="G28" s="5">
+        <f>IF($K28="","",INDEX(מלאי!$F$2:$F$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="H28" s="5">
+        <f>IF($K28="","",INDEX(מלאי!$AB$2:$AB$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="I28" s="4">
+        <f>IF($K28="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K28)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K28)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J28" s="4">
+        <f>IF($K28="","",INDEX(מלאי!$AC$2:$AC$500,$K28))</f>
+        <v/>
+      </c>
+      <c r="K28" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2">
+        <f>IF($K29="","",INDEX(מלאי!$D$2:$D$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="B29" s="2">
+        <f>IF($K29="","",INDEX(מלאי!$B$2:$B$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="C29" s="2">
+        <f>IF($K29="","",INDEX(מלאי!$C$2:$C$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="D29" s="2">
+        <f>IF($K29="","",INDEX(מלאי!$Y$2:$Y$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="E29" s="2">
+        <f>IF($K29="","",INDEX(מלאי!$Z$2:$Z$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="F29" s="2">
+        <f>IF($K29="","",INDEX(מלאי!$AA$2:$AA$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="G29" s="3">
+        <f>IF($K29="","",INDEX(מלאי!$F$2:$F$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="H29" s="3">
+        <f>IF($K29="","",INDEX(מלאי!$AB$2:$AB$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="I29" s="2">
+        <f>IF($K29="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K29)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K29)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J29" s="2">
+        <f>IF($K29="","",INDEX(מלאי!$AC$2:$AC$500,$K29))</f>
+        <v/>
+      </c>
+      <c r="K29" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4">
+        <f>IF($K30="","",INDEX(מלאי!$D$2:$D$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="B30" s="4">
+        <f>IF($K30="","",INDEX(מלאי!$B$2:$B$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="C30" s="4">
+        <f>IF($K30="","",INDEX(מלאי!$C$2:$C$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="D30" s="4">
+        <f>IF($K30="","",INDEX(מלאי!$Y$2:$Y$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="E30" s="4">
+        <f>IF($K30="","",INDEX(מלאי!$Z$2:$Z$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="F30" s="4">
+        <f>IF($K30="","",INDEX(מלאי!$AA$2:$AA$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="G30" s="5">
+        <f>IF($K30="","",INDEX(מלאי!$F$2:$F$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="H30" s="5">
+        <f>IF($K30="","",INDEX(מלאי!$AB$2:$AB$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="I30" s="4">
+        <f>IF($K30="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K30)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K30)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J30" s="4">
+        <f>IF($K30="","",INDEX(מלאי!$AC$2:$AC$500,$K30))</f>
+        <v/>
+      </c>
+      <c r="K30" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2">
+        <f>IF($K31="","",INDEX(מלאי!$D$2:$D$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="B31" s="2">
+        <f>IF($K31="","",INDEX(מלאי!$B$2:$B$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="C31" s="2">
+        <f>IF($K31="","",INDEX(מלאי!$C$2:$C$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="D31" s="2">
+        <f>IF($K31="","",INDEX(מלאי!$Y$2:$Y$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="E31" s="2">
+        <f>IF($K31="","",INDEX(מלאי!$Z$2:$Z$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="F31" s="2">
+        <f>IF($K31="","",INDEX(מלאי!$AA$2:$AA$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="G31" s="3">
+        <f>IF($K31="","",INDEX(מלאי!$F$2:$F$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="H31" s="3">
+        <f>IF($K31="","",INDEX(מלאי!$AB$2:$AB$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="I31" s="2">
+        <f>IF($K31="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K31)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K31)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J31" s="2">
+        <f>IF($K31="","",INDEX(מלאי!$AC$2:$AC$500,$K31))</f>
+        <v/>
+      </c>
+      <c r="K31" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4">
+        <f>IF($K32="","",INDEX(מלאי!$D$2:$D$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="B32" s="4">
+        <f>IF($K32="","",INDEX(מלאי!$B$2:$B$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="C32" s="4">
+        <f>IF($K32="","",INDEX(מלאי!$C$2:$C$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="D32" s="4">
+        <f>IF($K32="","",INDEX(מלאי!$Y$2:$Y$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="E32" s="4">
+        <f>IF($K32="","",INDEX(מלאי!$Z$2:$Z$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="F32" s="4">
+        <f>IF($K32="","",INDEX(מלאי!$AA$2:$AA$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="G32" s="5">
+        <f>IF($K32="","",INDEX(מלאי!$F$2:$F$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="H32" s="5">
+        <f>IF($K32="","",INDEX(מלאי!$AB$2:$AB$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="I32" s="4">
+        <f>IF($K32="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K32)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K32)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J32" s="4">
+        <f>IF($K32="","",INDEX(מלאי!$AC$2:$AC$500,$K32))</f>
+        <v/>
+      </c>
+      <c r="K32" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),28),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2">
+        <f>IF($K33="","",INDEX(מלאי!$D$2:$D$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="B33" s="2">
+        <f>IF($K33="","",INDEX(מלאי!$B$2:$B$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="C33" s="2">
+        <f>IF($K33="","",INDEX(מלאי!$C$2:$C$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="D33" s="2">
+        <f>IF($K33="","",INDEX(מלאי!$Y$2:$Y$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="E33" s="2">
+        <f>IF($K33="","",INDEX(מלאי!$Z$2:$Z$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="F33" s="2">
+        <f>IF($K33="","",INDEX(מלאי!$AA$2:$AA$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="G33" s="3">
+        <f>IF($K33="","",INDEX(מלאי!$F$2:$F$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="H33" s="3">
+        <f>IF($K33="","",INDEX(מלאי!$AB$2:$AB$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="I33" s="2">
+        <f>IF($K33="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K33)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K33)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J33" s="2">
+        <f>IF($K33="","",INDEX(מלאי!$AC$2:$AC$500,$K33))</f>
+        <v/>
+      </c>
+      <c r="K33" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),29),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4">
+        <f>IF($K34="","",INDEX(מלאי!$D$2:$D$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="B34" s="4">
+        <f>IF($K34="","",INDEX(מלאי!$B$2:$B$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="C34" s="4">
+        <f>IF($K34="","",INDEX(מלאי!$C$2:$C$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="D34" s="4">
+        <f>IF($K34="","",INDEX(מלאי!$Y$2:$Y$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="E34" s="4">
+        <f>IF($K34="","",INDEX(מלאי!$Z$2:$Z$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="F34" s="4">
+        <f>IF($K34="","",INDEX(מלאי!$AA$2:$AA$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="G34" s="5">
+        <f>IF($K34="","",INDEX(מלאי!$F$2:$F$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="H34" s="5">
+        <f>IF($K34="","",INDEX(מלאי!$AB$2:$AB$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="I34" s="4">
+        <f>IF($K34="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K34)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K34)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J34" s="4">
+        <f>IF($K34="","",INDEX(מלאי!$AC$2:$AC$500,$K34))</f>
+        <v/>
+      </c>
+      <c r="K34" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),30),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2">
+        <f>IF($K35="","",INDEX(מלאי!$D$2:$D$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="B35" s="2">
+        <f>IF($K35="","",INDEX(מלאי!$B$2:$B$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="C35" s="2">
+        <f>IF($K35="","",INDEX(מלאי!$C$2:$C$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="D35" s="2">
+        <f>IF($K35="","",INDEX(מלאי!$Y$2:$Y$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="E35" s="2">
+        <f>IF($K35="","",INDEX(מלאי!$Z$2:$Z$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="F35" s="2">
+        <f>IF($K35="","",INDEX(מלאי!$AA$2:$AA$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="G35" s="3">
+        <f>IF($K35="","",INDEX(מלאי!$F$2:$F$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="H35" s="3">
+        <f>IF($K35="","",INDEX(מלאי!$AB$2:$AB$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="I35" s="2">
+        <f>IF($K35="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K35)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K35)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J35" s="2">
+        <f>IF($K35="","",INDEX(מלאי!$AC$2:$AC$500,$K35))</f>
+        <v/>
+      </c>
+      <c r="K35" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),31),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4">
+        <f>IF($K36="","",INDEX(מלאי!$D$2:$D$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="B36" s="4">
+        <f>IF($K36="","",INDEX(מלאי!$B$2:$B$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="C36" s="4">
+        <f>IF($K36="","",INDEX(מלאי!$C$2:$C$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="D36" s="4">
+        <f>IF($K36="","",INDEX(מלאי!$Y$2:$Y$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="E36" s="4">
+        <f>IF($K36="","",INDEX(מלאי!$Z$2:$Z$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="F36" s="4">
+        <f>IF($K36="","",INDEX(מלאי!$AA$2:$AA$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="G36" s="5">
+        <f>IF($K36="","",INDEX(מלאי!$F$2:$F$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="H36" s="5">
+        <f>IF($K36="","",INDEX(מלאי!$AB$2:$AB$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="I36" s="4">
+        <f>IF($K36="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K36)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K36)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J36" s="4">
+        <f>IF($K36="","",INDEX(מלאי!$AC$2:$AC$500,$K36))</f>
+        <v/>
+      </c>
+      <c r="K36" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),32),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2">
+        <f>IF($K37="","",INDEX(מלאי!$D$2:$D$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="B37" s="2">
+        <f>IF($K37="","",INDEX(מלאי!$B$2:$B$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="C37" s="2">
+        <f>IF($K37="","",INDEX(מלאי!$C$2:$C$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="D37" s="2">
+        <f>IF($K37="","",INDEX(מלאי!$Y$2:$Y$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="E37" s="2">
+        <f>IF($K37="","",INDEX(מלאי!$Z$2:$Z$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="F37" s="2">
+        <f>IF($K37="","",INDEX(מלאי!$AA$2:$AA$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="G37" s="3">
+        <f>IF($K37="","",INDEX(מלאי!$F$2:$F$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="H37" s="3">
+        <f>IF($K37="","",INDEX(מלאי!$AB$2:$AB$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="I37" s="2">
+        <f>IF($K37="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K37)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K37)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J37" s="2">
+        <f>IF($K37="","",INDEX(מלאי!$AC$2:$AC$500,$K37))</f>
+        <v/>
+      </c>
+      <c r="K37" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),33),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4">
+        <f>IF($K38="","",INDEX(מלאי!$D$2:$D$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="B38" s="4">
+        <f>IF($K38="","",INDEX(מלאי!$B$2:$B$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="C38" s="4">
+        <f>IF($K38="","",INDEX(מלאי!$C$2:$C$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="D38" s="4">
+        <f>IF($K38="","",INDEX(מלאי!$Y$2:$Y$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="E38" s="4">
+        <f>IF($K38="","",INDEX(מלאי!$Z$2:$Z$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="F38" s="4">
+        <f>IF($K38="","",INDEX(מלאי!$AA$2:$AA$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="G38" s="5">
+        <f>IF($K38="","",INDEX(מלאי!$F$2:$F$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="H38" s="5">
+        <f>IF($K38="","",INDEX(מלאי!$AB$2:$AB$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="I38" s="4">
+        <f>IF($K38="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K38)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K38)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J38" s="4">
+        <f>IF($K38="","",INDEX(מלאי!$AC$2:$AC$500,$K38))</f>
+        <v/>
+      </c>
+      <c r="K38" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),34),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2">
+        <f>IF($K39="","",INDEX(מלאי!$D$2:$D$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="B39" s="2">
+        <f>IF($K39="","",INDEX(מלאי!$B$2:$B$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="C39" s="2">
+        <f>IF($K39="","",INDEX(מלאי!$C$2:$C$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="D39" s="2">
+        <f>IF($K39="","",INDEX(מלאי!$Y$2:$Y$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="E39" s="2">
+        <f>IF($K39="","",INDEX(מלאי!$Z$2:$Z$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="F39" s="2">
+        <f>IF($K39="","",INDEX(מלאי!$AA$2:$AA$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="G39" s="3">
+        <f>IF($K39="","",INDEX(מלאי!$F$2:$F$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="H39" s="3">
+        <f>IF($K39="","",INDEX(מלאי!$AB$2:$AB$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="I39" s="2">
+        <f>IF($K39="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K39)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K39)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J39" s="2">
+        <f>IF($K39="","",INDEX(מלאי!$AC$2:$AC$500,$K39))</f>
+        <v/>
+      </c>
+      <c r="K39" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),35),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4">
+        <f>IF($K40="","",INDEX(מלאי!$D$2:$D$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="B40" s="4">
+        <f>IF($K40="","",INDEX(מלאי!$B$2:$B$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="C40" s="4">
+        <f>IF($K40="","",INDEX(מלאי!$C$2:$C$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="D40" s="4">
+        <f>IF($K40="","",INDEX(מלאי!$Y$2:$Y$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="E40" s="4">
+        <f>IF($K40="","",INDEX(מלאי!$Z$2:$Z$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="F40" s="4">
+        <f>IF($K40="","",INDEX(מלאי!$AA$2:$AA$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="G40" s="5">
+        <f>IF($K40="","",INDEX(מלאי!$F$2:$F$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="H40" s="5">
+        <f>IF($K40="","",INDEX(מלאי!$AB$2:$AB$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="I40" s="4">
+        <f>IF($K40="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K40)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K40)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J40" s="4">
+        <f>IF($K40="","",INDEX(מלאי!$AC$2:$AC$500,$K40))</f>
+        <v/>
+      </c>
+      <c r="K40" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),36),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2">
+        <f>IF($K41="","",INDEX(מלאי!$D$2:$D$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="B41" s="2">
+        <f>IF($K41="","",INDEX(מלאי!$B$2:$B$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="C41" s="2">
+        <f>IF($K41="","",INDEX(מלאי!$C$2:$C$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="D41" s="2">
+        <f>IF($K41="","",INDEX(מלאי!$Y$2:$Y$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="E41" s="2">
+        <f>IF($K41="","",INDEX(מלאי!$Z$2:$Z$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="F41" s="2">
+        <f>IF($K41="","",INDEX(מלאי!$AA$2:$AA$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="G41" s="3">
+        <f>IF($K41="","",INDEX(מלאי!$F$2:$F$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="H41" s="3">
+        <f>IF($K41="","",INDEX(מלאי!$AB$2:$AB$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="I41" s="2">
+        <f>IF($K41="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K41)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K41)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J41" s="2">
+        <f>IF($K41="","",INDEX(מלאי!$AC$2:$AC$500,$K41))</f>
+        <v/>
+      </c>
+      <c r="K41" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),37),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4">
+        <f>IF($K42="","",INDEX(מלאי!$D$2:$D$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="B42" s="4">
+        <f>IF($K42="","",INDEX(מלאי!$B$2:$B$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="C42" s="4">
+        <f>IF($K42="","",INDEX(מלאי!$C$2:$C$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="D42" s="4">
+        <f>IF($K42="","",INDEX(מלאי!$Y$2:$Y$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="E42" s="4">
+        <f>IF($K42="","",INDEX(מלאי!$Z$2:$Z$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="F42" s="4">
+        <f>IF($K42="","",INDEX(מלאי!$AA$2:$AA$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="G42" s="5">
+        <f>IF($K42="","",INDEX(מלאי!$F$2:$F$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="H42" s="5">
+        <f>IF($K42="","",INDEX(מלאי!$AB$2:$AB$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="I42" s="4">
+        <f>IF($K42="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K42)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K42)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J42" s="4">
+        <f>IF($K42="","",INDEX(מלאי!$AC$2:$AC$500,$K42))</f>
+        <v/>
+      </c>
+      <c r="K42" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),38),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2">
+        <f>IF($K43="","",INDEX(מלאי!$D$2:$D$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="B43" s="2">
+        <f>IF($K43="","",INDEX(מלאי!$B$2:$B$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="C43" s="2">
+        <f>IF($K43="","",INDEX(מלאי!$C$2:$C$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="D43" s="2">
+        <f>IF($K43="","",INDEX(מלאי!$Y$2:$Y$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="E43" s="2">
+        <f>IF($K43="","",INDEX(מלאי!$Z$2:$Z$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="F43" s="2">
+        <f>IF($K43="","",INDEX(מלאי!$AA$2:$AA$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="G43" s="3">
+        <f>IF($K43="","",INDEX(מלאי!$F$2:$F$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="H43" s="3">
+        <f>IF($K43="","",INDEX(מלאי!$AB$2:$AB$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="I43" s="2">
+        <f>IF($K43="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K43)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K43)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J43" s="2">
+        <f>IF($K43="","",INDEX(מלאי!$AC$2:$AC$500,$K43))</f>
+        <v/>
+      </c>
+      <c r="K43" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),39),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4">
+        <f>IF($K44="","",INDEX(מלאי!$D$2:$D$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="B44" s="4">
+        <f>IF($K44="","",INDEX(מלאי!$B$2:$B$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="C44" s="4">
+        <f>IF($K44="","",INDEX(מלאי!$C$2:$C$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="D44" s="4">
+        <f>IF($K44="","",INDEX(מלאי!$Y$2:$Y$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="E44" s="4">
+        <f>IF($K44="","",INDEX(מלאי!$Z$2:$Z$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="F44" s="4">
+        <f>IF($K44="","",INDEX(מלאי!$AA$2:$AA$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="G44" s="5">
+        <f>IF($K44="","",INDEX(מלאי!$F$2:$F$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="H44" s="5">
+        <f>IF($K44="","",INDEX(מלאי!$AB$2:$AB$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="I44" s="4">
+        <f>IF($K44="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K44)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K44)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J44" s="4">
+        <f>IF($K44="","",INDEX(מלאי!$AC$2:$AC$500,$K44))</f>
+        <v/>
+      </c>
+      <c r="K44" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),40),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2">
+        <f>IF($K45="","",INDEX(מלאי!$D$2:$D$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="B45" s="2">
+        <f>IF($K45="","",INDEX(מלאי!$B$2:$B$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="C45" s="2">
+        <f>IF($K45="","",INDEX(מלאי!$C$2:$C$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="D45" s="2">
+        <f>IF($K45="","",INDEX(מלאי!$Y$2:$Y$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="E45" s="2">
+        <f>IF($K45="","",INDEX(מלאי!$Z$2:$Z$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="F45" s="2">
+        <f>IF($K45="","",INDEX(מלאי!$AA$2:$AA$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="G45" s="3">
+        <f>IF($K45="","",INDEX(מלאי!$F$2:$F$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="H45" s="3">
+        <f>IF($K45="","",INDEX(מלאי!$AB$2:$AB$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="I45" s="2">
+        <f>IF($K45="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K45)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K45)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J45" s="2">
+        <f>IF($K45="","",INDEX(מלאי!$AC$2:$AC$500,$K45))</f>
+        <v/>
+      </c>
+      <c r="K45" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),41),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4">
+        <f>IF($K46="","",INDEX(מלאי!$D$2:$D$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="B46" s="4">
+        <f>IF($K46="","",INDEX(מלאי!$B$2:$B$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="C46" s="4">
+        <f>IF($K46="","",INDEX(מלאי!$C$2:$C$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="D46" s="4">
+        <f>IF($K46="","",INDEX(מלאי!$Y$2:$Y$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="E46" s="4">
+        <f>IF($K46="","",INDEX(מלאי!$Z$2:$Z$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="F46" s="4">
+        <f>IF($K46="","",INDEX(מלאי!$AA$2:$AA$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="G46" s="5">
+        <f>IF($K46="","",INDEX(מלאי!$F$2:$F$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="H46" s="5">
+        <f>IF($K46="","",INDEX(מלאי!$AB$2:$AB$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="I46" s="4">
+        <f>IF($K46="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K46)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K46)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J46" s="4">
+        <f>IF($K46="","",INDEX(מלאי!$AC$2:$AC$500,$K46))</f>
+        <v/>
+      </c>
+      <c r="K46" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),42),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2">
+        <f>IF($K47="","",INDEX(מלאי!$D$2:$D$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="B47" s="2">
+        <f>IF($K47="","",INDEX(מלאי!$B$2:$B$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="C47" s="2">
+        <f>IF($K47="","",INDEX(מלאי!$C$2:$C$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="D47" s="2">
+        <f>IF($K47="","",INDEX(מלאי!$Y$2:$Y$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="E47" s="2">
+        <f>IF($K47="","",INDEX(מלאי!$Z$2:$Z$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="F47" s="2">
+        <f>IF($K47="","",INDEX(מלאי!$AA$2:$AA$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="G47" s="3">
+        <f>IF($K47="","",INDEX(מלאי!$F$2:$F$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="H47" s="3">
+        <f>IF($K47="","",INDEX(מלאי!$AB$2:$AB$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="I47" s="2">
+        <f>IF($K47="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K47)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K47)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J47" s="2">
+        <f>IF($K47="","",INDEX(מלאי!$AC$2:$AC$500,$K47))</f>
+        <v/>
+      </c>
+      <c r="K47" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),43),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4">
+        <f>IF($K48="","",INDEX(מלאי!$D$2:$D$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="B48" s="4">
+        <f>IF($K48="","",INDEX(מלאי!$B$2:$B$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="C48" s="4">
+        <f>IF($K48="","",INDEX(מלאי!$C$2:$C$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="D48" s="4">
+        <f>IF($K48="","",INDEX(מלאי!$Y$2:$Y$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="E48" s="4">
+        <f>IF($K48="","",INDEX(מלאי!$Z$2:$Z$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="F48" s="4">
+        <f>IF($K48="","",INDEX(מלאי!$AA$2:$AA$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="G48" s="5">
+        <f>IF($K48="","",INDEX(מלאי!$F$2:$F$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="H48" s="5">
+        <f>IF($K48="","",INDEX(מלאי!$AB$2:$AB$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="I48" s="4">
+        <f>IF($K48="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K48)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K48)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J48" s="4">
+        <f>IF($K48="","",INDEX(מלאי!$AC$2:$AC$500,$K48))</f>
+        <v/>
+      </c>
+      <c r="K48" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),44),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2">
+        <f>IF($K49="","",INDEX(מלאי!$D$2:$D$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="B49" s="2">
+        <f>IF($K49="","",INDEX(מלאי!$B$2:$B$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="C49" s="2">
+        <f>IF($K49="","",INDEX(מלאי!$C$2:$C$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="D49" s="2">
+        <f>IF($K49="","",INDEX(מלאי!$Y$2:$Y$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="E49" s="2">
+        <f>IF($K49="","",INDEX(מלאי!$Z$2:$Z$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="F49" s="2">
+        <f>IF($K49="","",INDEX(מלאי!$AA$2:$AA$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="G49" s="3">
+        <f>IF($K49="","",INDEX(מלאי!$F$2:$F$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="H49" s="3">
+        <f>IF($K49="","",INDEX(מלאי!$AB$2:$AB$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="I49" s="2">
+        <f>IF($K49="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K49)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K49)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J49" s="2">
+        <f>IF($K49="","",INDEX(מלאי!$AC$2:$AC$500,$K49))</f>
+        <v/>
+      </c>
+      <c r="K49" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),45),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4">
+        <f>IF($K50="","",INDEX(מלאי!$D$2:$D$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="B50" s="4">
+        <f>IF($K50="","",INDEX(מלאי!$B$2:$B$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="C50" s="4">
+        <f>IF($K50="","",INDEX(מלאי!$C$2:$C$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="D50" s="4">
+        <f>IF($K50="","",INDEX(מלאי!$Y$2:$Y$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="E50" s="4">
+        <f>IF($K50="","",INDEX(מלאי!$Z$2:$Z$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="F50" s="4">
+        <f>IF($K50="","",INDEX(מלאי!$AA$2:$AA$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="G50" s="5">
+        <f>IF($K50="","",INDEX(מלאי!$F$2:$F$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="H50" s="5">
+        <f>IF($K50="","",INDEX(מלאי!$AB$2:$AB$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="I50" s="4">
+        <f>IF($K50="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K50)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K50)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J50" s="4">
+        <f>IF($K50="","",INDEX(מלאי!$AC$2:$AC$500,$K50))</f>
+        <v/>
+      </c>
+      <c r="K50" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),46),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2">
+        <f>IF($K51="","",INDEX(מלאי!$D$2:$D$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="B51" s="2">
+        <f>IF($K51="","",INDEX(מלאי!$B$2:$B$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="C51" s="2">
+        <f>IF($K51="","",INDEX(מלאי!$C$2:$C$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="D51" s="2">
+        <f>IF($K51="","",INDEX(מלאי!$Y$2:$Y$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="E51" s="2">
+        <f>IF($K51="","",INDEX(מלאי!$Z$2:$Z$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="F51" s="2">
+        <f>IF($K51="","",INDEX(מלאי!$AA$2:$AA$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="G51" s="3">
+        <f>IF($K51="","",INDEX(מלאי!$F$2:$F$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="H51" s="3">
+        <f>IF($K51="","",INDEX(מלאי!$AB$2:$AB$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="I51" s="2">
+        <f>IF($K51="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K51)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K51)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J51" s="2">
+        <f>IF($K51="","",INDEX(מלאי!$AC$2:$AC$500,$K51))</f>
+        <v/>
+      </c>
+      <c r="K51" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),47),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4">
+        <f>IF($K52="","",INDEX(מלאי!$D$2:$D$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="B52" s="4">
+        <f>IF($K52="","",INDEX(מלאי!$B$2:$B$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="C52" s="4">
+        <f>IF($K52="","",INDEX(מלאי!$C$2:$C$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="D52" s="4">
+        <f>IF($K52="","",INDEX(מלאי!$Y$2:$Y$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="E52" s="4">
+        <f>IF($K52="","",INDEX(מלאי!$Z$2:$Z$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="F52" s="4">
+        <f>IF($K52="","",INDEX(מלאי!$AA$2:$AA$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="G52" s="5">
+        <f>IF($K52="","",INDEX(מלאי!$F$2:$F$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="H52" s="5">
+        <f>IF($K52="","",INDEX(מלאי!$AB$2:$AB$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="I52" s="4">
+        <f>IF($K52="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K52)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K52)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J52" s="4">
+        <f>IF($K52="","",INDEX(מלאי!$AC$2:$AC$500,$K52))</f>
+        <v/>
+      </c>
+      <c r="K52" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),48),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2">
+        <f>IF($K53="","",INDEX(מלאי!$D$2:$D$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="B53" s="2">
+        <f>IF($K53="","",INDEX(מלאי!$B$2:$B$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="C53" s="2">
+        <f>IF($K53="","",INDEX(מלאי!$C$2:$C$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="D53" s="2">
+        <f>IF($K53="","",INDEX(מלאי!$Y$2:$Y$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="E53" s="2">
+        <f>IF($K53="","",INDEX(מלאי!$Z$2:$Z$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="F53" s="2">
+        <f>IF($K53="","",INDEX(מלאי!$AA$2:$AA$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="G53" s="3">
+        <f>IF($K53="","",INDEX(מלאי!$F$2:$F$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="H53" s="3">
+        <f>IF($K53="","",INDEX(מלאי!$AB$2:$AB$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="I53" s="2">
+        <f>IF($K53="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K53)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K53)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J53" s="2">
+        <f>IF($K53="","",INDEX(מלאי!$AC$2:$AC$500,$K53))</f>
+        <v/>
+      </c>
+      <c r="K53" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),49),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4">
+        <f>IF($K54="","",INDEX(מלאי!$D$2:$D$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="B54" s="4">
+        <f>IF($K54="","",INDEX(מלאי!$B$2:$B$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="C54" s="4">
+        <f>IF($K54="","",INDEX(מלאי!$C$2:$C$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="D54" s="4">
+        <f>IF($K54="","",INDEX(מלאי!$Y$2:$Y$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="E54" s="4">
+        <f>IF($K54="","",INDEX(מלאי!$Z$2:$Z$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="F54" s="4">
+        <f>IF($K54="","",INDEX(מלאי!$AA$2:$AA$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="G54" s="5">
+        <f>IF($K54="","",INDEX(מלאי!$F$2:$F$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="H54" s="5">
+        <f>IF($K54="","",INDEX(מלאי!$AB$2:$AB$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="I54" s="4">
+        <f>IF($K54="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K54)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K54)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J54" s="4">
+        <f>IF($K54="","",INDEX(מלאי!$AC$2:$AC$500,$K54))</f>
+        <v/>
+      </c>
+      <c r="K54" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),50),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2">
+        <f>IF($K55="","",INDEX(מלאי!$D$2:$D$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="B55" s="2">
+        <f>IF($K55="","",INDEX(מלאי!$B$2:$B$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="C55" s="2">
+        <f>IF($K55="","",INDEX(מלאי!$C$2:$C$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="D55" s="2">
+        <f>IF($K55="","",INDEX(מלאי!$Y$2:$Y$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="E55" s="2">
+        <f>IF($K55="","",INDEX(מלאי!$Z$2:$Z$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="F55" s="2">
+        <f>IF($K55="","",INDEX(מלאי!$AA$2:$AA$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="G55" s="3">
+        <f>IF($K55="","",INDEX(מלאי!$F$2:$F$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="H55" s="3">
+        <f>IF($K55="","",INDEX(מלאי!$AB$2:$AB$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="I55" s="2">
+        <f>IF($K55="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K55)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K55)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J55" s="2">
+        <f>IF($K55="","",INDEX(מלאי!$AC$2:$AC$500,$K55))</f>
+        <v/>
+      </c>
+      <c r="K55" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),51),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4">
+        <f>IF($K56="","",INDEX(מלאי!$D$2:$D$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="B56" s="4">
+        <f>IF($K56="","",INDEX(מלאי!$B$2:$B$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="C56" s="4">
+        <f>IF($K56="","",INDEX(מלאי!$C$2:$C$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="D56" s="4">
+        <f>IF($K56="","",INDEX(מלאי!$Y$2:$Y$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="E56" s="4">
+        <f>IF($K56="","",INDEX(מלאי!$Z$2:$Z$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="F56" s="4">
+        <f>IF($K56="","",INDEX(מלאי!$AA$2:$AA$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="G56" s="5">
+        <f>IF($K56="","",INDEX(מלאי!$F$2:$F$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="H56" s="5">
+        <f>IF($K56="","",INDEX(מלאי!$AB$2:$AB$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="I56" s="4">
+        <f>IF($K56="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K56)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K56)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J56" s="4">
+        <f>IF($K56="","",INDEX(מלאי!$AC$2:$AC$500,$K56))</f>
+        <v/>
+      </c>
+      <c r="K56" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),52),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2">
+        <f>IF($K57="","",INDEX(מלאי!$D$2:$D$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="B57" s="2">
+        <f>IF($K57="","",INDEX(מלאי!$B$2:$B$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="C57" s="2">
+        <f>IF($K57="","",INDEX(מלאי!$C$2:$C$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="D57" s="2">
+        <f>IF($K57="","",INDEX(מלאי!$Y$2:$Y$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="E57" s="2">
+        <f>IF($K57="","",INDEX(מלאי!$Z$2:$Z$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="F57" s="2">
+        <f>IF($K57="","",INDEX(מלאי!$AA$2:$AA$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="G57" s="3">
+        <f>IF($K57="","",INDEX(מלאי!$F$2:$F$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="H57" s="3">
+        <f>IF($K57="","",INDEX(מלאי!$AB$2:$AB$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="I57" s="2">
+        <f>IF($K57="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K57)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K57)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J57" s="2">
+        <f>IF($K57="","",INDEX(מלאי!$AC$2:$AC$500,$K57))</f>
+        <v/>
+      </c>
+      <c r="K57" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),53),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4">
+        <f>IF($K58="","",INDEX(מלאי!$D$2:$D$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="B58" s="4">
+        <f>IF($K58="","",INDEX(מלאי!$B$2:$B$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="C58" s="4">
+        <f>IF($K58="","",INDEX(מלאי!$C$2:$C$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="D58" s="4">
+        <f>IF($K58="","",INDEX(מלאי!$Y$2:$Y$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="E58" s="4">
+        <f>IF($K58="","",INDEX(מלאי!$Z$2:$Z$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="F58" s="4">
+        <f>IF($K58="","",INDEX(מלאי!$AA$2:$AA$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="G58" s="5">
+        <f>IF($K58="","",INDEX(מלאי!$F$2:$F$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="H58" s="5">
+        <f>IF($K58="","",INDEX(מלאי!$AB$2:$AB$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="I58" s="4">
+        <f>IF($K58="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K58)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K58)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J58" s="4">
+        <f>IF($K58="","",INDEX(מלאי!$AC$2:$AC$500,$K58))</f>
+        <v/>
+      </c>
+      <c r="K58" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),54),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2">
+        <f>IF($K59="","",INDEX(מלאי!$D$2:$D$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="B59" s="2">
+        <f>IF($K59="","",INDEX(מלאי!$B$2:$B$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="C59" s="2">
+        <f>IF($K59="","",INDEX(מלאי!$C$2:$C$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="D59" s="2">
+        <f>IF($K59="","",INDEX(מלאי!$Y$2:$Y$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="E59" s="2">
+        <f>IF($K59="","",INDEX(מלאי!$Z$2:$Z$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="F59" s="2">
+        <f>IF($K59="","",INDEX(מלאי!$AA$2:$AA$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="G59" s="3">
+        <f>IF($K59="","",INDEX(מלאי!$F$2:$F$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="H59" s="3">
+        <f>IF($K59="","",INDEX(מלאי!$AB$2:$AB$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="I59" s="2">
+        <f>IF($K59="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K59)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K59)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J59" s="2">
+        <f>IF($K59="","",INDEX(מלאי!$AC$2:$AC$500,$K59))</f>
+        <v/>
+      </c>
+      <c r="K59" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),55),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4">
+        <f>IF($K60="","",INDEX(מלאי!$D$2:$D$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="B60" s="4">
+        <f>IF($K60="","",INDEX(מלאי!$B$2:$B$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="C60" s="4">
+        <f>IF($K60="","",INDEX(מלאי!$C$2:$C$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="D60" s="4">
+        <f>IF($K60="","",INDEX(מלאי!$Y$2:$Y$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="E60" s="4">
+        <f>IF($K60="","",INDEX(מלאי!$Z$2:$Z$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="F60" s="4">
+        <f>IF($K60="","",INDEX(מלאי!$AA$2:$AA$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="G60" s="5">
+        <f>IF($K60="","",INDEX(מלאי!$F$2:$F$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="H60" s="5">
+        <f>IF($K60="","",INDEX(מלאי!$AB$2:$AB$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="I60" s="4">
+        <f>IF($K60="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K60)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K60)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J60" s="4">
+        <f>IF($K60="","",INDEX(מלאי!$AC$2:$AC$500,$K60))</f>
+        <v/>
+      </c>
+      <c r="K60" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),56),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2">
+        <f>IF($K61="","",INDEX(מלאי!$D$2:$D$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="B61" s="2">
+        <f>IF($K61="","",INDEX(מלאי!$B$2:$B$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="C61" s="2">
+        <f>IF($K61="","",INDEX(מלאי!$C$2:$C$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="D61" s="2">
+        <f>IF($K61="","",INDEX(מלאי!$Y$2:$Y$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="E61" s="2">
+        <f>IF($K61="","",INDEX(מלאי!$Z$2:$Z$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="F61" s="2">
+        <f>IF($K61="","",INDEX(מלאי!$AA$2:$AA$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="G61" s="3">
+        <f>IF($K61="","",INDEX(מלאי!$F$2:$F$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="H61" s="3">
+        <f>IF($K61="","",INDEX(מלאי!$AB$2:$AB$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="I61" s="2">
+        <f>IF($K61="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K61)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K61)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J61" s="2">
+        <f>IF($K61="","",INDEX(מלאי!$AC$2:$AC$500,$K61))</f>
+        <v/>
+      </c>
+      <c r="K61" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),57),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4">
+        <f>IF($K62="","",INDEX(מלאי!$D$2:$D$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="B62" s="4">
+        <f>IF($K62="","",INDEX(מלאי!$B$2:$B$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="C62" s="4">
+        <f>IF($K62="","",INDEX(מלאי!$C$2:$C$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="D62" s="4">
+        <f>IF($K62="","",INDEX(מלאי!$Y$2:$Y$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="E62" s="4">
+        <f>IF($K62="","",INDEX(מלאי!$Z$2:$Z$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="F62" s="4">
+        <f>IF($K62="","",INDEX(מלאי!$AA$2:$AA$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="G62" s="5">
+        <f>IF($K62="","",INDEX(מלאי!$F$2:$F$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="H62" s="5">
+        <f>IF($K62="","",INDEX(מלאי!$AB$2:$AB$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="I62" s="4">
+        <f>IF($K62="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K62)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K62)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J62" s="4">
+        <f>IF($K62="","",INDEX(מלאי!$AC$2:$AC$500,$K62))</f>
+        <v/>
+      </c>
+      <c r="K62" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),58),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2">
+        <f>IF($K63="","",INDEX(מלאי!$D$2:$D$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="B63" s="2">
+        <f>IF($K63="","",INDEX(מלאי!$B$2:$B$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="C63" s="2">
+        <f>IF($K63="","",INDEX(מלאי!$C$2:$C$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="D63" s="2">
+        <f>IF($K63="","",INDEX(מלאי!$Y$2:$Y$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="E63" s="2">
+        <f>IF($K63="","",INDEX(מלאי!$Z$2:$Z$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="F63" s="2">
+        <f>IF($K63="","",INDEX(מלאי!$AA$2:$AA$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="G63" s="3">
+        <f>IF($K63="","",INDEX(מלאי!$F$2:$F$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="H63" s="3">
+        <f>IF($K63="","",INDEX(מלאי!$AB$2:$AB$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="I63" s="2">
+        <f>IF($K63="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K63)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K63)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J63" s="2">
+        <f>IF($K63="","",INDEX(מלאי!$AC$2:$AC$500,$K63))</f>
+        <v/>
+      </c>
+      <c r="K63" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),59),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4">
+        <f>IF($K64="","",INDEX(מלאי!$D$2:$D$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="B64" s="4">
+        <f>IF($K64="","",INDEX(מלאי!$B$2:$B$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="C64" s="4">
+        <f>IF($K64="","",INDEX(מלאי!$C$2:$C$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="D64" s="4">
+        <f>IF($K64="","",INDEX(מלאי!$Y$2:$Y$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="E64" s="4">
+        <f>IF($K64="","",INDEX(מלאי!$Z$2:$Z$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="F64" s="4">
+        <f>IF($K64="","",INDEX(מלאי!$AA$2:$AA$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="G64" s="5">
+        <f>IF($K64="","",INDEX(מלאי!$F$2:$F$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="H64" s="5">
+        <f>IF($K64="","",INDEX(מלאי!$AB$2:$AB$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="I64" s="4">
+        <f>IF($K64="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K64)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K64)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J64" s="4">
+        <f>IF($K64="","",INDEX(מלאי!$AC$2:$AC$500,$K64))</f>
+        <v/>
+      </c>
+      <c r="K64" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),60),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2">
+        <f>IF($K65="","",INDEX(מלאי!$D$2:$D$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="B65" s="2">
+        <f>IF($K65="","",INDEX(מלאי!$B$2:$B$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="C65" s="2">
+        <f>IF($K65="","",INDEX(מלאי!$C$2:$C$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="D65" s="2">
+        <f>IF($K65="","",INDEX(מלאי!$Y$2:$Y$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="E65" s="2">
+        <f>IF($K65="","",INDEX(מלאי!$Z$2:$Z$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="F65" s="2">
+        <f>IF($K65="","",INDEX(מלאי!$AA$2:$AA$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="G65" s="3">
+        <f>IF($K65="","",INDEX(מלאי!$F$2:$F$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="H65" s="3">
+        <f>IF($K65="","",INDEX(מלאי!$AB$2:$AB$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="I65" s="2">
+        <f>IF($K65="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K65)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K65)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J65" s="2">
+        <f>IF($K65="","",INDEX(מלאי!$AC$2:$AC$500,$K65))</f>
+        <v/>
+      </c>
+      <c r="K65" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),61),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4">
+        <f>IF($K66="","",INDEX(מלאי!$D$2:$D$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="B66" s="4">
+        <f>IF($K66="","",INDEX(מלאי!$B$2:$B$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="C66" s="4">
+        <f>IF($K66="","",INDEX(מלאי!$C$2:$C$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="D66" s="4">
+        <f>IF($K66="","",INDEX(מלאי!$Y$2:$Y$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="E66" s="4">
+        <f>IF($K66="","",INDEX(מלאי!$Z$2:$Z$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="F66" s="4">
+        <f>IF($K66="","",INDEX(מלאי!$AA$2:$AA$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="G66" s="5">
+        <f>IF($K66="","",INDEX(מלאי!$F$2:$F$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="H66" s="5">
+        <f>IF($K66="","",INDEX(מלאי!$AB$2:$AB$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="I66" s="4">
+        <f>IF($K66="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K66)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K66)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J66" s="4">
+        <f>IF($K66="","",INDEX(מלאי!$AC$2:$AC$500,$K66))</f>
+        <v/>
+      </c>
+      <c r="K66" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),62),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2">
+        <f>IF($K67="","",INDEX(מלאי!$D$2:$D$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="B67" s="2">
+        <f>IF($K67="","",INDEX(מלאי!$B$2:$B$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="C67" s="2">
+        <f>IF($K67="","",INDEX(מלאי!$C$2:$C$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="D67" s="2">
+        <f>IF($K67="","",INDEX(מלאי!$Y$2:$Y$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="E67" s="2">
+        <f>IF($K67="","",INDEX(מלאי!$Z$2:$Z$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="F67" s="2">
+        <f>IF($K67="","",INDEX(מלאי!$AA$2:$AA$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="G67" s="3">
+        <f>IF($K67="","",INDEX(מלאי!$F$2:$F$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="H67" s="3">
+        <f>IF($K67="","",INDEX(מלאי!$AB$2:$AB$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="I67" s="2">
+        <f>IF($K67="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K67)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K67)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J67" s="2">
+        <f>IF($K67="","",INDEX(מלאי!$AC$2:$AC$500,$K67))</f>
+        <v/>
+      </c>
+      <c r="K67" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),63),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4">
+        <f>IF($K68="","",INDEX(מלאי!$D$2:$D$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="B68" s="4">
+        <f>IF($K68="","",INDEX(מלאי!$B$2:$B$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="C68" s="4">
+        <f>IF($K68="","",INDEX(מלאי!$C$2:$C$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="D68" s="4">
+        <f>IF($K68="","",INDEX(מלאי!$Y$2:$Y$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="E68" s="4">
+        <f>IF($K68="","",INDEX(מלאי!$Z$2:$Z$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="F68" s="4">
+        <f>IF($K68="","",INDEX(מלאי!$AA$2:$AA$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="G68" s="5">
+        <f>IF($K68="","",INDEX(מלאי!$F$2:$F$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="H68" s="5">
+        <f>IF($K68="","",INDEX(מלאי!$AB$2:$AB$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="I68" s="4">
+        <f>IF($K68="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K68)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K68)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J68" s="4">
+        <f>IF($K68="","",INDEX(מלאי!$AC$2:$AC$500,$K68))</f>
+        <v/>
+      </c>
+      <c r="K68" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),64),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2">
+        <f>IF($K69="","",INDEX(מלאי!$D$2:$D$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="B69" s="2">
+        <f>IF($K69="","",INDEX(מלאי!$B$2:$B$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="C69" s="2">
+        <f>IF($K69="","",INDEX(מלאי!$C$2:$C$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="D69" s="2">
+        <f>IF($K69="","",INDEX(מלאי!$Y$2:$Y$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="E69" s="2">
+        <f>IF($K69="","",INDEX(מלאי!$Z$2:$Z$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="F69" s="2">
+        <f>IF($K69="","",INDEX(מלאי!$AA$2:$AA$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="G69" s="3">
+        <f>IF($K69="","",INDEX(מלאי!$F$2:$F$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="H69" s="3">
+        <f>IF($K69="","",INDEX(מלאי!$AB$2:$AB$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="I69" s="2">
+        <f>IF($K69="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K69)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K69)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J69" s="2">
+        <f>IF($K69="","",INDEX(מלאי!$AC$2:$AC$500,$K69))</f>
+        <v/>
+      </c>
+      <c r="K69" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),65),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4">
+        <f>IF($K70="","",INDEX(מלאי!$D$2:$D$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="B70" s="4">
+        <f>IF($K70="","",INDEX(מלאי!$B$2:$B$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="C70" s="4">
+        <f>IF($K70="","",INDEX(מלאי!$C$2:$C$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="D70" s="4">
+        <f>IF($K70="","",INDEX(מלאי!$Y$2:$Y$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="E70" s="4">
+        <f>IF($K70="","",INDEX(מלאי!$Z$2:$Z$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="F70" s="4">
+        <f>IF($K70="","",INDEX(מלאי!$AA$2:$AA$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="G70" s="5">
+        <f>IF($K70="","",INDEX(מלאי!$F$2:$F$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="H70" s="5">
+        <f>IF($K70="","",INDEX(מלאי!$AB$2:$AB$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="I70" s="4">
+        <f>IF($K70="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K70)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K70)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J70" s="4">
+        <f>IF($K70="","",INDEX(מלאי!$AC$2:$AC$500,$K70))</f>
+        <v/>
+      </c>
+      <c r="K70" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),66),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2">
+        <f>IF($K71="","",INDEX(מלאי!$D$2:$D$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="B71" s="2">
+        <f>IF($K71="","",INDEX(מלאי!$B$2:$B$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="C71" s="2">
+        <f>IF($K71="","",INDEX(מלאי!$C$2:$C$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="D71" s="2">
+        <f>IF($K71="","",INDEX(מלאי!$Y$2:$Y$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="E71" s="2">
+        <f>IF($K71="","",INDEX(מלאי!$Z$2:$Z$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="F71" s="2">
+        <f>IF($K71="","",INDEX(מלאי!$AA$2:$AA$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="G71" s="3">
+        <f>IF($K71="","",INDEX(מלאי!$F$2:$F$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="H71" s="3">
+        <f>IF($K71="","",INDEX(מלאי!$AB$2:$AB$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="I71" s="2">
+        <f>IF($K71="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K71)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K71)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J71" s="2">
+        <f>IF($K71="","",INDEX(מלאי!$AC$2:$AC$500,$K71))</f>
+        <v/>
+      </c>
+      <c r="K71" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),67),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4">
+        <f>IF($K72="","",INDEX(מלאי!$D$2:$D$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="B72" s="4">
+        <f>IF($K72="","",INDEX(מלאי!$B$2:$B$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="C72" s="4">
+        <f>IF($K72="","",INDEX(מלאי!$C$2:$C$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="D72" s="4">
+        <f>IF($K72="","",INDEX(מלאי!$Y$2:$Y$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="E72" s="4">
+        <f>IF($K72="","",INDEX(מלאי!$Z$2:$Z$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="F72" s="4">
+        <f>IF($K72="","",INDEX(מלאי!$AA$2:$AA$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="G72" s="5">
+        <f>IF($K72="","",INDEX(מלאי!$F$2:$F$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="H72" s="5">
+        <f>IF($K72="","",INDEX(מלאי!$AB$2:$AB$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="I72" s="4">
+        <f>IF($K72="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K72)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K72)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J72" s="4">
+        <f>IF($K72="","",INDEX(מלאי!$AC$2:$AC$500,$K72))</f>
+        <v/>
+      </c>
+      <c r="K72" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),68),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2">
+        <f>IF($K73="","",INDEX(מלאי!$D$2:$D$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="B73" s="2">
+        <f>IF($K73="","",INDEX(מלאי!$B$2:$B$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="C73" s="2">
+        <f>IF($K73="","",INDEX(מלאי!$C$2:$C$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="D73" s="2">
+        <f>IF($K73="","",INDEX(מלאי!$Y$2:$Y$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="E73" s="2">
+        <f>IF($K73="","",INDEX(מלאי!$Z$2:$Z$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="F73" s="2">
+        <f>IF($K73="","",INDEX(מלאי!$AA$2:$AA$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="G73" s="3">
+        <f>IF($K73="","",INDEX(מלאי!$F$2:$F$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="H73" s="3">
+        <f>IF($K73="","",INDEX(מלאי!$AB$2:$AB$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="I73" s="2">
+        <f>IF($K73="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K73)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K73)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J73" s="2">
+        <f>IF($K73="","",INDEX(מלאי!$AC$2:$AC$500,$K73))</f>
+        <v/>
+      </c>
+      <c r="K73" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),69),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4">
+        <f>IF($K74="","",INDEX(מלאי!$D$2:$D$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="B74" s="4">
+        <f>IF($K74="","",INDEX(מלאי!$B$2:$B$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="C74" s="4">
+        <f>IF($K74="","",INDEX(מלאי!$C$2:$C$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="D74" s="4">
+        <f>IF($K74="","",INDEX(מלאי!$Y$2:$Y$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="E74" s="4">
+        <f>IF($K74="","",INDEX(מלאי!$Z$2:$Z$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="F74" s="4">
+        <f>IF($K74="","",INDEX(מלאי!$AA$2:$AA$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="G74" s="5">
+        <f>IF($K74="","",INDEX(מלאי!$F$2:$F$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="H74" s="5">
+        <f>IF($K74="","",INDEX(מלאי!$AB$2:$AB$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="I74" s="4">
+        <f>IF($K74="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K74)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K74)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J74" s="4">
+        <f>IF($K74="","",INDEX(מלאי!$AC$2:$AC$500,$K74))</f>
+        <v/>
+      </c>
+      <c r="K74" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),70),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2">
+        <f>IF($K75="","",INDEX(מלאי!$D$2:$D$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="B75" s="2">
+        <f>IF($K75="","",INDEX(מלאי!$B$2:$B$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="C75" s="2">
+        <f>IF($K75="","",INDEX(מלאי!$C$2:$C$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="D75" s="2">
+        <f>IF($K75="","",INDEX(מלאי!$Y$2:$Y$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="E75" s="2">
+        <f>IF($K75="","",INDEX(מלאי!$Z$2:$Z$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="F75" s="2">
+        <f>IF($K75="","",INDEX(מלאי!$AA$2:$AA$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="G75" s="3">
+        <f>IF($K75="","",INDEX(מלאי!$F$2:$F$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="H75" s="3">
+        <f>IF($K75="","",INDEX(מלאי!$AB$2:$AB$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="I75" s="2">
+        <f>IF($K75="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K75)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K75)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J75" s="2">
+        <f>IF($K75="","",INDEX(מלאי!$AC$2:$AC$500,$K75))</f>
+        <v/>
+      </c>
+      <c r="K75" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),71),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4">
+        <f>IF($K76="","",INDEX(מלאי!$D$2:$D$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="B76" s="4">
+        <f>IF($K76="","",INDEX(מלאי!$B$2:$B$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="C76" s="4">
+        <f>IF($K76="","",INDEX(מלאי!$C$2:$C$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="D76" s="4">
+        <f>IF($K76="","",INDEX(מלאי!$Y$2:$Y$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="E76" s="4">
+        <f>IF($K76="","",INDEX(מלאי!$Z$2:$Z$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="F76" s="4">
+        <f>IF($K76="","",INDEX(מלאי!$AA$2:$AA$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="G76" s="5">
+        <f>IF($K76="","",INDEX(מלאי!$F$2:$F$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="H76" s="5">
+        <f>IF($K76="","",INDEX(מלאי!$AB$2:$AB$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="I76" s="4">
+        <f>IF($K76="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K76)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K76)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J76" s="4">
+        <f>IF($K76="","",INDEX(מלאי!$AC$2:$AC$500,$K76))</f>
+        <v/>
+      </c>
+      <c r="K76" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),72),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2">
+        <f>IF($K77="","",INDEX(מלאי!$D$2:$D$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="B77" s="2">
+        <f>IF($K77="","",INDEX(מלאי!$B$2:$B$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="C77" s="2">
+        <f>IF($K77="","",INDEX(מלאי!$C$2:$C$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="D77" s="2">
+        <f>IF($K77="","",INDEX(מלאי!$Y$2:$Y$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="E77" s="2">
+        <f>IF($K77="","",INDEX(מלאי!$Z$2:$Z$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="F77" s="2">
+        <f>IF($K77="","",INDEX(מלאי!$AA$2:$AA$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="G77" s="3">
+        <f>IF($K77="","",INDEX(מלאי!$F$2:$F$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="H77" s="3">
+        <f>IF($K77="","",INDEX(מלאי!$AB$2:$AB$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="I77" s="2">
+        <f>IF($K77="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K77)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K77)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J77" s="2">
+        <f>IF($K77="","",INDEX(מלאי!$AC$2:$AC$500,$K77))</f>
+        <v/>
+      </c>
+      <c r="K77" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),73),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4">
+        <f>IF($K78="","",INDEX(מלאי!$D$2:$D$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="B78" s="4">
+        <f>IF($K78="","",INDEX(מלאי!$B$2:$B$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="C78" s="4">
+        <f>IF($K78="","",INDEX(מלאי!$C$2:$C$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="D78" s="4">
+        <f>IF($K78="","",INDEX(מלאי!$Y$2:$Y$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="E78" s="4">
+        <f>IF($K78="","",INDEX(מלאי!$Z$2:$Z$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="F78" s="4">
+        <f>IF($K78="","",INDEX(מלאי!$AA$2:$AA$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="G78" s="5">
+        <f>IF($K78="","",INDEX(מלאי!$F$2:$F$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="H78" s="5">
+        <f>IF($K78="","",INDEX(מלאי!$AB$2:$AB$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="I78" s="4">
+        <f>IF($K78="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K78)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K78)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J78" s="4">
+        <f>IF($K78="","",INDEX(מלאי!$AC$2:$AC$500,$K78))</f>
+        <v/>
+      </c>
+      <c r="K78" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),74),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2">
+        <f>IF($K79="","",INDEX(מלאי!$D$2:$D$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="B79" s="2">
+        <f>IF($K79="","",INDEX(מלאי!$B$2:$B$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="C79" s="2">
+        <f>IF($K79="","",INDEX(מלאי!$C$2:$C$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="D79" s="2">
+        <f>IF($K79="","",INDEX(מלאי!$Y$2:$Y$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="E79" s="2">
+        <f>IF($K79="","",INDEX(מלאי!$Z$2:$Z$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="F79" s="2">
+        <f>IF($K79="","",INDEX(מלאי!$AA$2:$AA$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="G79" s="3">
+        <f>IF($K79="","",INDEX(מלאי!$F$2:$F$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="H79" s="3">
+        <f>IF($K79="","",INDEX(מלאי!$AB$2:$AB$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="I79" s="2">
+        <f>IF($K79="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K79)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K79)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J79" s="2">
+        <f>IF($K79="","",INDEX(מלאי!$AC$2:$AC$500,$K79))</f>
+        <v/>
+      </c>
+      <c r="K79" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),75),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4">
+        <f>IF($K80="","",INDEX(מלאי!$D$2:$D$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="B80" s="4">
+        <f>IF($K80="","",INDEX(מלאי!$B$2:$B$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="C80" s="4">
+        <f>IF($K80="","",INDEX(מלאי!$C$2:$C$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="D80" s="4">
+        <f>IF($K80="","",INDEX(מלאי!$Y$2:$Y$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="E80" s="4">
+        <f>IF($K80="","",INDEX(מלאי!$Z$2:$Z$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="F80" s="4">
+        <f>IF($K80="","",INDEX(מלאי!$AA$2:$AA$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="G80" s="5">
+        <f>IF($K80="","",INDEX(מלאי!$F$2:$F$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="H80" s="5">
+        <f>IF($K80="","",INDEX(מלאי!$AB$2:$AB$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="I80" s="4">
+        <f>IF($K80="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K80)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K80)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J80" s="4">
+        <f>IF($K80="","",INDEX(מלאי!$AC$2:$AC$500,$K80))</f>
+        <v/>
+      </c>
+      <c r="K80" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),76),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2">
+        <f>IF($K81="","",INDEX(מלאי!$D$2:$D$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="B81" s="2">
+        <f>IF($K81="","",INDEX(מלאי!$B$2:$B$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="C81" s="2">
+        <f>IF($K81="","",INDEX(מלאי!$C$2:$C$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="D81" s="2">
+        <f>IF($K81="","",INDEX(מלאי!$Y$2:$Y$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="E81" s="2">
+        <f>IF($K81="","",INDEX(מלאי!$Z$2:$Z$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="F81" s="2">
+        <f>IF($K81="","",INDEX(מלאי!$AA$2:$AA$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="G81" s="3">
+        <f>IF($K81="","",INDEX(מלאי!$F$2:$F$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="H81" s="3">
+        <f>IF($K81="","",INDEX(מלאי!$AB$2:$AB$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="I81" s="2">
+        <f>IF($K81="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K81)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K81)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J81" s="2">
+        <f>IF($K81="","",INDEX(מלאי!$AC$2:$AC$500,$K81))</f>
+        <v/>
+      </c>
+      <c r="K81" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),77),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4">
+        <f>IF($K82="","",INDEX(מלאי!$D$2:$D$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="B82" s="4">
+        <f>IF($K82="","",INDEX(מלאי!$B$2:$B$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="C82" s="4">
+        <f>IF($K82="","",INDEX(מלאי!$C$2:$C$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="D82" s="4">
+        <f>IF($K82="","",INDEX(מלאי!$Y$2:$Y$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="E82" s="4">
+        <f>IF($K82="","",INDEX(מלאי!$Z$2:$Z$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="F82" s="4">
+        <f>IF($K82="","",INDEX(מלאי!$AA$2:$AA$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="G82" s="5">
+        <f>IF($K82="","",INDEX(מלאי!$F$2:$F$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="H82" s="5">
+        <f>IF($K82="","",INDEX(מלאי!$AB$2:$AB$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="I82" s="4">
+        <f>IF($K82="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K82)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K82)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J82" s="4">
+        <f>IF($K82="","",INDEX(מלאי!$AC$2:$AC$500,$K82))</f>
+        <v/>
+      </c>
+      <c r="K82" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),78),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2">
+        <f>IF($K83="","",INDEX(מלאי!$D$2:$D$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="B83" s="2">
+        <f>IF($K83="","",INDEX(מלאי!$B$2:$B$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="C83" s="2">
+        <f>IF($K83="","",INDEX(מלאי!$C$2:$C$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="D83" s="2">
+        <f>IF($K83="","",INDEX(מלאי!$Y$2:$Y$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="E83" s="2">
+        <f>IF($K83="","",INDEX(מלאי!$Z$2:$Z$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="F83" s="2">
+        <f>IF($K83="","",INDEX(מלאי!$AA$2:$AA$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="G83" s="3">
+        <f>IF($K83="","",INDEX(מלאי!$F$2:$F$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="H83" s="3">
+        <f>IF($K83="","",INDEX(מלאי!$AB$2:$AB$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="I83" s="2">
+        <f>IF($K83="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K83)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K83)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J83" s="2">
+        <f>IF($K83="","",INDEX(מלאי!$AC$2:$AC$500,$K83))</f>
+        <v/>
+      </c>
+      <c r="K83" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),79),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4">
+        <f>IF($K84="","",INDEX(מלאי!$D$2:$D$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="B84" s="4">
+        <f>IF($K84="","",INDEX(מלאי!$B$2:$B$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="C84" s="4">
+        <f>IF($K84="","",INDEX(מלאי!$C$2:$C$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="D84" s="4">
+        <f>IF($K84="","",INDEX(מלאי!$Y$2:$Y$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="E84" s="4">
+        <f>IF($K84="","",INDEX(מלאי!$Z$2:$Z$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="F84" s="4">
+        <f>IF($K84="","",INDEX(מלאי!$AA$2:$AA$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="G84" s="5">
+        <f>IF($K84="","",INDEX(מלאי!$F$2:$F$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="H84" s="5">
+        <f>IF($K84="","",INDEX(מלאי!$AB$2:$AB$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="I84" s="4">
+        <f>IF($K84="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K84)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K84)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J84" s="4">
+        <f>IF($K84="","",INDEX(מלאי!$AC$2:$AC$500,$K84))</f>
+        <v/>
+      </c>
+      <c r="K84" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),80),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2">
+        <f>IF($K85="","",INDEX(מלאי!$D$2:$D$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="B85" s="2">
+        <f>IF($K85="","",INDEX(מלאי!$B$2:$B$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="C85" s="2">
+        <f>IF($K85="","",INDEX(מלאי!$C$2:$C$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="D85" s="2">
+        <f>IF($K85="","",INDEX(מלאי!$Y$2:$Y$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="E85" s="2">
+        <f>IF($K85="","",INDEX(מלאי!$Z$2:$Z$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="F85" s="2">
+        <f>IF($K85="","",INDEX(מלאי!$AA$2:$AA$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="G85" s="3">
+        <f>IF($K85="","",INDEX(מלאי!$F$2:$F$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="H85" s="3">
+        <f>IF($K85="","",INDEX(מלאי!$AB$2:$AB$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="I85" s="2">
+        <f>IF($K85="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K85)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K85)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J85" s="2">
+        <f>IF($K85="","",INDEX(מלאי!$AC$2:$AC$500,$K85))</f>
+        <v/>
+      </c>
+      <c r="K85" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),81),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4">
+        <f>IF($K86="","",INDEX(מלאי!$D$2:$D$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="B86" s="4">
+        <f>IF($K86="","",INDEX(מלאי!$B$2:$B$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="C86" s="4">
+        <f>IF($K86="","",INDEX(מלאי!$C$2:$C$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="D86" s="4">
+        <f>IF($K86="","",INDEX(מלאי!$Y$2:$Y$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="E86" s="4">
+        <f>IF($K86="","",INDEX(מלאי!$Z$2:$Z$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="F86" s="4">
+        <f>IF($K86="","",INDEX(מלאי!$AA$2:$AA$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="G86" s="5">
+        <f>IF($K86="","",INDEX(מלאי!$F$2:$F$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="H86" s="5">
+        <f>IF($K86="","",INDEX(מלאי!$AB$2:$AB$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="I86" s="4">
+        <f>IF($K86="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K86)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K86)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J86" s="4">
+        <f>IF($K86="","",INDEX(מלאי!$AC$2:$AC$500,$K86))</f>
+        <v/>
+      </c>
+      <c r="K86" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),82),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2">
+        <f>IF($K87="","",INDEX(מלאי!$D$2:$D$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="B87" s="2">
+        <f>IF($K87="","",INDEX(מלאי!$B$2:$B$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="C87" s="2">
+        <f>IF($K87="","",INDEX(מלאי!$C$2:$C$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="D87" s="2">
+        <f>IF($K87="","",INDEX(מלאי!$Y$2:$Y$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="E87" s="2">
+        <f>IF($K87="","",INDEX(מלאי!$Z$2:$Z$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="F87" s="2">
+        <f>IF($K87="","",INDEX(מלאי!$AA$2:$AA$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="G87" s="3">
+        <f>IF($K87="","",INDEX(מלאי!$F$2:$F$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="H87" s="3">
+        <f>IF($K87="","",INDEX(מלאי!$AB$2:$AB$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="I87" s="2">
+        <f>IF($K87="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K87)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K87)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J87" s="2">
+        <f>IF($K87="","",INDEX(מלאי!$AC$2:$AC$500,$K87))</f>
+        <v/>
+      </c>
+      <c r="K87" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),83),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4">
+        <f>IF($K88="","",INDEX(מלאי!$D$2:$D$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="B88" s="4">
+        <f>IF($K88="","",INDEX(מלאי!$B$2:$B$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="C88" s="4">
+        <f>IF($K88="","",INDEX(מלאי!$C$2:$C$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="D88" s="4">
+        <f>IF($K88="","",INDEX(מלאי!$Y$2:$Y$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="E88" s="4">
+        <f>IF($K88="","",INDEX(מלאי!$Z$2:$Z$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="F88" s="4">
+        <f>IF($K88="","",INDEX(מלאי!$AA$2:$AA$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="G88" s="5">
+        <f>IF($K88="","",INDEX(מלאי!$F$2:$F$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="H88" s="5">
+        <f>IF($K88="","",INDEX(מלאי!$AB$2:$AB$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="I88" s="4">
+        <f>IF($K88="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K88)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K88)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J88" s="4">
+        <f>IF($K88="","",INDEX(מלאי!$AC$2:$AC$500,$K88))</f>
+        <v/>
+      </c>
+      <c r="K88" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),84),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2">
+        <f>IF($K89="","",INDEX(מלאי!$D$2:$D$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="B89" s="2">
+        <f>IF($K89="","",INDEX(מלאי!$B$2:$B$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="C89" s="2">
+        <f>IF($K89="","",INDEX(מלאי!$C$2:$C$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="D89" s="2">
+        <f>IF($K89="","",INDEX(מלאי!$Y$2:$Y$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="E89" s="2">
+        <f>IF($K89="","",INDEX(מלאי!$Z$2:$Z$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="F89" s="2">
+        <f>IF($K89="","",INDEX(מלאי!$AA$2:$AA$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="G89" s="3">
+        <f>IF($K89="","",INDEX(מלאי!$F$2:$F$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="H89" s="3">
+        <f>IF($K89="","",INDEX(מלאי!$AB$2:$AB$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="I89" s="2">
+        <f>IF($K89="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K89)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K89)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J89" s="2">
+        <f>IF($K89="","",INDEX(מלאי!$AC$2:$AC$500,$K89))</f>
+        <v/>
+      </c>
+      <c r="K89" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),85),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4">
+        <f>IF($K90="","",INDEX(מלאי!$D$2:$D$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="B90" s="4">
+        <f>IF($K90="","",INDEX(מלאי!$B$2:$B$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="C90" s="4">
+        <f>IF($K90="","",INDEX(מלאי!$C$2:$C$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="D90" s="4">
+        <f>IF($K90="","",INDEX(מלאי!$Y$2:$Y$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="E90" s="4">
+        <f>IF($K90="","",INDEX(מלאי!$Z$2:$Z$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="F90" s="4">
+        <f>IF($K90="","",INDEX(מלאי!$AA$2:$AA$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="G90" s="5">
+        <f>IF($K90="","",INDEX(מלאי!$F$2:$F$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="H90" s="5">
+        <f>IF($K90="","",INDEX(מלאי!$AB$2:$AB$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="I90" s="4">
+        <f>IF($K90="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K90)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K90)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J90" s="4">
+        <f>IF($K90="","",INDEX(מלאי!$AC$2:$AC$500,$K90))</f>
+        <v/>
+      </c>
+      <c r="K90" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),86),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2">
+        <f>IF($K91="","",INDEX(מלאי!$D$2:$D$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="B91" s="2">
+        <f>IF($K91="","",INDEX(מלאי!$B$2:$B$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="C91" s="2">
+        <f>IF($K91="","",INDEX(מלאי!$C$2:$C$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="D91" s="2">
+        <f>IF($K91="","",INDEX(מלאי!$Y$2:$Y$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="E91" s="2">
+        <f>IF($K91="","",INDEX(מלאי!$Z$2:$Z$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="F91" s="2">
+        <f>IF($K91="","",INDEX(מלאי!$AA$2:$AA$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="G91" s="3">
+        <f>IF($K91="","",INDEX(מלאי!$F$2:$F$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="H91" s="3">
+        <f>IF($K91="","",INDEX(מלאי!$AB$2:$AB$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="I91" s="2">
+        <f>IF($K91="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K91)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K91)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J91" s="2">
+        <f>IF($K91="","",INDEX(מלאי!$AC$2:$AC$500,$K91))</f>
+        <v/>
+      </c>
+      <c r="K91" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),87),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4">
+        <f>IF($K92="","",INDEX(מלאי!$D$2:$D$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="B92" s="4">
+        <f>IF($K92="","",INDEX(מלאי!$B$2:$B$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="C92" s="4">
+        <f>IF($K92="","",INDEX(מלאי!$C$2:$C$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="D92" s="4">
+        <f>IF($K92="","",INDEX(מלאי!$Y$2:$Y$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="E92" s="4">
+        <f>IF($K92="","",INDEX(מלאי!$Z$2:$Z$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="F92" s="4">
+        <f>IF($K92="","",INDEX(מלאי!$AA$2:$AA$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="G92" s="5">
+        <f>IF($K92="","",INDEX(מלאי!$F$2:$F$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="H92" s="5">
+        <f>IF($K92="","",INDEX(מלאי!$AB$2:$AB$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="I92" s="4">
+        <f>IF($K92="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K92)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K92)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J92" s="4">
+        <f>IF($K92="","",INDEX(מלאי!$AC$2:$AC$500,$K92))</f>
+        <v/>
+      </c>
+      <c r="K92" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),88),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2">
+        <f>IF($K93="","",INDEX(מלאי!$D$2:$D$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="B93" s="2">
+        <f>IF($K93="","",INDEX(מלאי!$B$2:$B$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="C93" s="2">
+        <f>IF($K93="","",INDEX(מלאי!$C$2:$C$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="D93" s="2">
+        <f>IF($K93="","",INDEX(מלאי!$Y$2:$Y$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="E93" s="2">
+        <f>IF($K93="","",INDEX(מלאי!$Z$2:$Z$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="F93" s="2">
+        <f>IF($K93="","",INDEX(מלאי!$AA$2:$AA$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="G93" s="3">
+        <f>IF($K93="","",INDEX(מלאי!$F$2:$F$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="H93" s="3">
+        <f>IF($K93="","",INDEX(מלאי!$AB$2:$AB$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="I93" s="2">
+        <f>IF($K93="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K93)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K93)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J93" s="2">
+        <f>IF($K93="","",INDEX(מלאי!$AC$2:$AC$500,$K93))</f>
+        <v/>
+      </c>
+      <c r="K93" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),89),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4">
+        <f>IF($K94="","",INDEX(מלאי!$D$2:$D$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="B94" s="4">
+        <f>IF($K94="","",INDEX(מלאי!$B$2:$B$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="C94" s="4">
+        <f>IF($K94="","",INDEX(מלאי!$C$2:$C$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="D94" s="4">
+        <f>IF($K94="","",INDEX(מלאי!$Y$2:$Y$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="E94" s="4">
+        <f>IF($K94="","",INDEX(מלאי!$Z$2:$Z$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="F94" s="4">
+        <f>IF($K94="","",INDEX(מלאי!$AA$2:$AA$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="G94" s="5">
+        <f>IF($K94="","",INDEX(מלאי!$F$2:$F$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="H94" s="5">
+        <f>IF($K94="","",INDEX(מלאי!$AB$2:$AB$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="I94" s="4">
+        <f>IF($K94="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K94)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K94)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J94" s="4">
+        <f>IF($K94="","",INDEX(מלאי!$AC$2:$AC$500,$K94))</f>
+        <v/>
+      </c>
+      <c r="K94" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),90),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2">
+        <f>IF($K95="","",INDEX(מלאי!$D$2:$D$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="B95" s="2">
+        <f>IF($K95="","",INDEX(מלאי!$B$2:$B$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="C95" s="2">
+        <f>IF($K95="","",INDEX(מלאי!$C$2:$C$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="D95" s="2">
+        <f>IF($K95="","",INDEX(מלאי!$Y$2:$Y$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="E95" s="2">
+        <f>IF($K95="","",INDEX(מלאי!$Z$2:$Z$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="F95" s="2">
+        <f>IF($K95="","",INDEX(מלאי!$AA$2:$AA$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="G95" s="3">
+        <f>IF($K95="","",INDEX(מלאי!$F$2:$F$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="H95" s="3">
+        <f>IF($K95="","",INDEX(מלאי!$AB$2:$AB$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="I95" s="2">
+        <f>IF($K95="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K95)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K95)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J95" s="2">
+        <f>IF($K95="","",INDEX(מלאי!$AC$2:$AC$500,$K95))</f>
+        <v/>
+      </c>
+      <c r="K95" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),91),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="4">
+        <f>IF($K96="","",INDEX(מלאי!$D$2:$D$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="B96" s="4">
+        <f>IF($K96="","",INDEX(מלאי!$B$2:$B$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="C96" s="4">
+        <f>IF($K96="","",INDEX(מלאי!$C$2:$C$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="D96" s="4">
+        <f>IF($K96="","",INDEX(מלאי!$Y$2:$Y$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="E96" s="4">
+        <f>IF($K96="","",INDEX(מלאי!$Z$2:$Z$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="F96" s="4">
+        <f>IF($K96="","",INDEX(מלאי!$AA$2:$AA$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="G96" s="5">
+        <f>IF($K96="","",INDEX(מלאי!$F$2:$F$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="H96" s="5">
+        <f>IF($K96="","",INDEX(מלאי!$AB$2:$AB$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="I96" s="4">
+        <f>IF($K96="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K96)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K96)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J96" s="4">
+        <f>IF($K96="","",INDEX(מלאי!$AC$2:$AC$500,$K96))</f>
+        <v/>
+      </c>
+      <c r="K96" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),92),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2">
+        <f>IF($K97="","",INDEX(מלאי!$D$2:$D$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="B97" s="2">
+        <f>IF($K97="","",INDEX(מלאי!$B$2:$B$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="C97" s="2">
+        <f>IF($K97="","",INDEX(מלאי!$C$2:$C$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="D97" s="2">
+        <f>IF($K97="","",INDEX(מלאי!$Y$2:$Y$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="E97" s="2">
+        <f>IF($K97="","",INDEX(מלאי!$Z$2:$Z$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="F97" s="2">
+        <f>IF($K97="","",INDEX(מלאי!$AA$2:$AA$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="G97" s="3">
+        <f>IF($K97="","",INDEX(מלאי!$F$2:$F$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="H97" s="3">
+        <f>IF($K97="","",INDEX(מלאי!$AB$2:$AB$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="I97" s="2">
+        <f>IF($K97="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K97)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K97)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J97" s="2">
+        <f>IF($K97="","",INDEX(מלאי!$AC$2:$AC$500,$K97))</f>
+        <v/>
+      </c>
+      <c r="K97" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),93),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="4">
+        <f>IF($K98="","",INDEX(מלאי!$D$2:$D$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="B98" s="4">
+        <f>IF($K98="","",INDEX(מלאי!$B$2:$B$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="C98" s="4">
+        <f>IF($K98="","",INDEX(מלאי!$C$2:$C$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="D98" s="4">
+        <f>IF($K98="","",INDEX(מלאי!$Y$2:$Y$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="E98" s="4">
+        <f>IF($K98="","",INDEX(מלאי!$Z$2:$Z$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="F98" s="4">
+        <f>IF($K98="","",INDEX(מלאי!$AA$2:$AA$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="G98" s="5">
+        <f>IF($K98="","",INDEX(מלאי!$F$2:$F$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="H98" s="5">
+        <f>IF($K98="","",INDEX(מלאי!$AB$2:$AB$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="I98" s="4">
+        <f>IF($K98="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K98)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K98)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J98" s="4">
+        <f>IF($K98="","",INDEX(מלאי!$AC$2:$AC$500,$K98))</f>
+        <v/>
+      </c>
+      <c r="K98" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),94),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2">
+        <f>IF($K99="","",INDEX(מלאי!$D$2:$D$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="B99" s="2">
+        <f>IF($K99="","",INDEX(מלאי!$B$2:$B$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="C99" s="2">
+        <f>IF($K99="","",INDEX(מלאי!$C$2:$C$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="D99" s="2">
+        <f>IF($K99="","",INDEX(מלאי!$Y$2:$Y$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="E99" s="2">
+        <f>IF($K99="","",INDEX(מלאי!$Z$2:$Z$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="F99" s="2">
+        <f>IF($K99="","",INDEX(מלאי!$AA$2:$AA$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="G99" s="3">
+        <f>IF($K99="","",INDEX(מלאי!$F$2:$F$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="H99" s="3">
+        <f>IF($K99="","",INDEX(מלאי!$AB$2:$AB$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="I99" s="2">
+        <f>IF($K99="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K99)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K99)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J99" s="2">
+        <f>IF($K99="","",INDEX(מלאי!$AC$2:$AC$500,$K99))</f>
+        <v/>
+      </c>
+      <c r="K99" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),95),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="4">
+        <f>IF($K100="","",INDEX(מלאי!$D$2:$D$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="B100" s="4">
+        <f>IF($K100="","",INDEX(מלאי!$B$2:$B$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="C100" s="4">
+        <f>IF($K100="","",INDEX(מלאי!$C$2:$C$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="D100" s="4">
+        <f>IF($K100="","",INDEX(מלאי!$Y$2:$Y$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="E100" s="4">
+        <f>IF($K100="","",INDEX(מלאי!$Z$2:$Z$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="F100" s="4">
+        <f>IF($K100="","",INDEX(מלאי!$AA$2:$AA$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="G100" s="5">
+        <f>IF($K100="","",INDEX(מלאי!$F$2:$F$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="H100" s="5">
+        <f>IF($K100="","",INDEX(מלאי!$AB$2:$AB$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="I100" s="4">
+        <f>IF($K100="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K100)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K100)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J100" s="4">
+        <f>IF($K100="","",INDEX(מלאי!$AC$2:$AC$500,$K100))</f>
+        <v/>
+      </c>
+      <c r="K100" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),96),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2">
+        <f>IF($K101="","",INDEX(מלאי!$D$2:$D$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="B101" s="2">
+        <f>IF($K101="","",INDEX(מלאי!$B$2:$B$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="C101" s="2">
+        <f>IF($K101="","",INDEX(מלאי!$C$2:$C$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="D101" s="2">
+        <f>IF($K101="","",INDEX(מלאי!$Y$2:$Y$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="E101" s="2">
+        <f>IF($K101="","",INDEX(מלאי!$Z$2:$Z$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="F101" s="2">
+        <f>IF($K101="","",INDEX(מלאי!$AA$2:$AA$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="G101" s="3">
+        <f>IF($K101="","",INDEX(מלאי!$F$2:$F$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="H101" s="3">
+        <f>IF($K101="","",INDEX(מלאי!$AB$2:$AB$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="I101" s="2">
+        <f>IF($K101="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K101)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K101)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J101" s="2">
+        <f>IF($K101="","",INDEX(מלאי!$AC$2:$AC$500,$K101))</f>
+        <v/>
+      </c>
+      <c r="K101" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),97),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="4">
+        <f>IF($K102="","",INDEX(מלאי!$D$2:$D$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="B102" s="4">
+        <f>IF($K102="","",INDEX(מלאי!$B$2:$B$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="C102" s="4">
+        <f>IF($K102="","",INDEX(מלאי!$C$2:$C$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="D102" s="4">
+        <f>IF($K102="","",INDEX(מלאי!$Y$2:$Y$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="E102" s="4">
+        <f>IF($K102="","",INDEX(מלאי!$Z$2:$Z$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="F102" s="4">
+        <f>IF($K102="","",INDEX(מלאי!$AA$2:$AA$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="G102" s="5">
+        <f>IF($K102="","",INDEX(מלאי!$F$2:$F$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="H102" s="5">
+        <f>IF($K102="","",INDEX(מלאי!$AB$2:$AB$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="I102" s="4">
+        <f>IF($K102="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K102)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K102)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J102" s="4">
+        <f>IF($K102="","",INDEX(מלאי!$AC$2:$AC$500,$K102))</f>
+        <v/>
+      </c>
+      <c r="K102" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),98),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2">
+        <f>IF($K103="","",INDEX(מלאי!$D$2:$D$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="B103" s="2">
+        <f>IF($K103="","",INDEX(מלאי!$B$2:$B$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="C103" s="2">
+        <f>IF($K103="","",INDEX(מלאי!$C$2:$C$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="D103" s="2">
+        <f>IF($K103="","",INDEX(מלאי!$Y$2:$Y$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="E103" s="2">
+        <f>IF($K103="","",INDEX(מלאי!$Z$2:$Z$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="F103" s="2">
+        <f>IF($K103="","",INDEX(מלאי!$AA$2:$AA$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="G103" s="3">
+        <f>IF($K103="","",INDEX(מלאי!$F$2:$F$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="H103" s="3">
+        <f>IF($K103="","",INDEX(מלאי!$AB$2:$AB$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="I103" s="2">
+        <f>IF($K103="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K103)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K103)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J103" s="2">
+        <f>IF($K103="","",INDEX(מלאי!$AC$2:$AC$500,$K103))</f>
+        <v/>
+      </c>
+      <c r="K103" s="2">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),99),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4">
+        <f>IF($K104="","",INDEX(מלאי!$D$2:$D$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="B104" s="4">
+        <f>IF($K104="","",INDEX(מלאי!$B$2:$B$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="C104" s="4">
+        <f>IF($K104="","",INDEX(מלאי!$C$2:$C$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="D104" s="4">
+        <f>IF($K104="","",INDEX(מלאי!$Y$2:$Y$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="E104" s="4">
+        <f>IF($K104="","",INDEX(מלאי!$Z$2:$Z$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="F104" s="4">
+        <f>IF($K104="","",INDEX(מלאי!$AA$2:$AA$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="G104" s="5">
+        <f>IF($K104="","",INDEX(מלאי!$F$2:$F$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="H104" s="5">
+        <f>IF($K104="","",INDEX(מלאי!$AB$2:$AB$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="I104" s="4">
+        <f>IF($K104="","",IF(AND(INDEX(מלאי!$AB$2:$AB$500,$K104)&lt;&gt;"",INDEX(מלאי!$AB$2:$AB$500,$K104)&lt;TODAY()),"באיחור!","תקין"))</f>
+        <v/>
+      </c>
+      <c r="J104" s="4">
+        <f>IF($K104="","",INDEX(מלאי!$AC$2:$AC$500,$K104))</f>
+        <v/>
+      </c>
+      <c r="K104" s="4">
+        <f>IFERROR(SMALL(IF((מלאי!$X$2:$X$500="מושאל")*(IF($A$2="",1,מלאי!$Z$2:$Z$500=$A$2))*(IF($B$2="",1,מלאי!$Y$2:$Y$500=$B$2))*(IF($C$2="",1,מלאי!$AA$2:$AA$500=$C$2))*(IF($D$2="",1,IF($D$2="כן",(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY()),1-(מלאי!$AB$2:$AB$500&lt;&gt;"")*(מלאי!$AB$2:$AB$500&lt;TODAY())))),ROW(מלאי!$A$2:$A$500)-ROW(מלאי!$A$2)+1,""),100),"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="I5:I104">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>I5="באיחור!"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A5:J104">
+    <cfRule type="expression" priority="2" dxfId="2">
+      <formula>$I5="באיחור!"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="D2" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>כן_לא</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>